<commit_message>
Update Vilande kursplaner.xlsx with new analysis data
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/01 IIT/Analys/Vilande kursplaner.xlsx
+++ b/vault-dalarna-university/01 IIT/Analys/Vilande kursplaner.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Vilande kursplaner" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Vilande kursplaner'!$A$1:$H$87</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Vilande kursplaner'!$A$1:$I$87</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,17 +432,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H87"/>
+  <dimension ref="A1:I87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="58" customWidth="1" min="7" max="7"/>
-    <col width="70" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
+    <col width="58" customWidth="1" min="8" max="8"/>
+    <col width="70" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -468,20 +469,25 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Reviderad</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Ämnesnamn</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Kursnamn</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Problem</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Länk</t>
         </is>
@@ -508,22 +514,23 @@
           <t>2007-05-22</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
         <is>
           <t>Maskinteknik</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>3D CAD påbyggnad - Maskinteknik</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT2006</t>
         </is>
@@ -550,22 +557,23 @@
           <t>2007-06-13</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
         <is>
           <t>Informatik</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>Examensarbete för högskoleexamen i Informatik</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IK1032</t>
         </is>
@@ -592,22 +600,23 @@
           <t>2009-12-08</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
         <is>
           <t>Industriell ekonomi</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>Examensarbete för kandidatexamen i Industriell ekonomi</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IE2003</t>
         </is>
@@ -634,22 +643,23 @@
           <t>2013-02-21</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
         <is>
           <t>Byggteknik</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>Examensarbete i byggteknik för högskoleingenjörsexamen</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY2016</t>
         </is>
@@ -658,12 +668,12 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>IK1064</t>
+          <t>BY1047</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>BYA</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -673,39 +683,40 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2013-02-21</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Informatik</t>
-        </is>
-      </c>
+          <t>2013-03-14</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Datahantering och Problemlösning</t>
+          <t>Byggteknik</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IK1064</t>
+          <t>Bärkraftigt byggande och boende</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY1047</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>BY1047</t>
+          <t>IK1066</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>BYA</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -718,36 +729,37 @@
           <t>2013-03-14</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Byggteknik</t>
-        </is>
-      </c>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Bärkraftigt byggande och boende</t>
+          <t>Informatik</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY1047</t>
+          <t>Förändringsanalys</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IK1066</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>IK1066</t>
+          <t>MD1085</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -757,39 +769,40 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2013-03-14</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Informatik</t>
-        </is>
-      </c>
+          <t>2013-12-17</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Förändringsanalys</t>
+          <t>Matematikdidaktik</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IK1066</t>
+          <t>Matematikundervisning i ett specialpedagogiskt perspektiv</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD1085</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>MD1085</t>
+          <t>MT1060</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -799,39 +812,40 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2013-12-17</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Matematikdidaktik</t>
-        </is>
-      </c>
+          <t>2014-04-03</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Matematikundervisning i ett specialpedagogiskt perspektiv</t>
+          <t>Maskinteknik</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD1085</t>
+          <t>Hållfasthetslära</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1060</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>MT1060</t>
+          <t>IK1064</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -841,27 +855,32 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2014-04-03</t>
+          <t>2013-02-21</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Maskinteknik</t>
+          <t>2014-09-01</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Hållfasthetslära</t>
+          <t>Informatik</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1060</t>
+          <t>Datahantering och Problemlösning</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IK1064</t>
         </is>
       </c>
     </row>
@@ -886,22 +905,23 @@
           <t>2014-11-27</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
         <is>
           <t>Energiteknik</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>Examensarbete för masterexamen i solenergiteknik</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG4001</t>
         </is>
@@ -928,22 +948,23 @@
           <t>2015-03-05</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
         <is>
           <t>Matematikdidaktik</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>Matematikens historia för lärare</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD1097</t>
         </is>
@@ -970,22 +991,23 @@
           <t>2015-03-05</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr">
         <is>
           <t>Matematikdidaktik</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>Matematisk problemlösning i grundskolans senare år</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD1098</t>
         </is>
@@ -1012,22 +1034,23 @@
           <t>2015-03-20</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
         <is>
           <t>Byggteknik</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>Praktisk byggteknik</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY1059</t>
         </is>
@@ -1054,22 +1077,23 @@
           <t>2015-08-27</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
         <is>
           <t>Energiteknik</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>Solvärme</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3007</t>
         </is>
@@ -1096,22 +1120,23 @@
           <t>2015-08-27</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
         <is>
           <t>Energiteknik</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="G16" t="inlineStr">
         <is>
           <t>Solstrålning och solgeometri</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3015</t>
         </is>
@@ -1138,22 +1163,23 @@
           <t>2015-09-17</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
         <is>
           <t>Energiteknik</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="G17" t="inlineStr">
         <is>
           <t>Hållbara energisystem</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3012</t>
         </is>
@@ -1180,22 +1206,23 @@
           <t>2015-11-23</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
         <is>
           <t>Byggteknik</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="G18" t="inlineStr">
         <is>
           <t>Installationsteknik och dimensionering</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr">
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY1061</t>
         </is>
@@ -1222,22 +1249,23 @@
           <t>2016-03-24</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
         <is>
           <t>Matematik</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="G19" t="inlineStr">
         <is>
           <t>Matematik för tekniker</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="inlineStr">
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MA1040</t>
         </is>
@@ -1264,22 +1292,23 @@
           <t>2016-05-19</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
         <is>
           <t>Byggteknik</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="G20" t="inlineStr">
         <is>
           <t>Energiprojekt</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H20" s="2" t="inlineStr">
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY2022</t>
         </is>
@@ -1306,22 +1335,23 @@
           <t>2016-05-19</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr">
         <is>
           <t>Maskinteknik</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="G21" t="inlineStr">
         <is>
           <t>Introduktion till produktutveckling</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H21" s="2" t="inlineStr">
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1068</t>
         </is>
@@ -1348,22 +1378,23 @@
           <t>2016-09-01</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr">
         <is>
           <t>Byggteknik</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="G22" t="inlineStr">
         <is>
           <t>BIM projekt och projektering</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H22" s="2" t="inlineStr">
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY1065</t>
         </is>
@@ -1390,22 +1421,23 @@
           <t>2016-09-22</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr">
         <is>
           <t>Energiteknik</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="G23" t="inlineStr">
         <is>
           <t>Solenergiteknikpraktik</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H23" s="2" t="inlineStr">
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3017</t>
         </is>
@@ -1432,22 +1464,23 @@
           <t>2016-09-22</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr">
         <is>
           <t>Energiteknik</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="G24" t="inlineStr">
         <is>
           <t>Solenergiteknikpraktik</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H24" s="2" t="inlineStr">
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3018</t>
         </is>
@@ -1474,22 +1507,23 @@
           <t>2017-02-16</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr">
         <is>
           <t>Matematik</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
+      <c r="G25" t="inlineStr">
         <is>
           <t>Flervariabelanalys</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H25" s="2" t="inlineStr">
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MA1042</t>
         </is>
@@ -1516,22 +1550,23 @@
           <t>2017-10-12</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr">
         <is>
           <t>Samhällsbyggnadsteknik</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
+      <c r="G26" t="inlineStr">
         <is>
           <t>Vetenskapligt metod</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H26" s="2" t="inlineStr">
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SQ1003</t>
         </is>
@@ -1558,22 +1593,23 @@
           <t>2017-12-14</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr">
         <is>
           <t>Byggteknik</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
+      <c r="G27" t="inlineStr">
         <is>
           <t>Hållbar samhällsplanering</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H27" s="2" t="inlineStr">
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY3005</t>
         </is>
@@ -1600,22 +1636,23 @@
           <t>2018-02-15</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr">
         <is>
           <t>Maskinteknik</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
+      <c r="G28" t="inlineStr">
         <is>
           <t>Maskinelement</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H28" s="2" t="inlineStr">
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1074</t>
         </is>
@@ -1642,22 +1679,23 @@
           <t>2018-04-05</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr">
         <is>
           <t>Maskinteknik</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
+      <c r="G29" t="inlineStr">
         <is>
           <t>Produktutvecklingsmetoder</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H29" s="2" t="inlineStr">
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT228</t>
         </is>
@@ -1684,22 +1722,23 @@
           <t>2018-05-24</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr">
         <is>
           <t>Energiteknik</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr">
+      <c r="G30" t="inlineStr">
         <is>
           <t>Solenergins ekonomi</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H30" s="2" t="inlineStr">
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG225</t>
         </is>
@@ -1726,22 +1765,23 @@
           <t>2018-05-24</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr">
         <is>
           <t>Samhällsbyggnadsteknik</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="G31" t="inlineStr">
         <is>
           <t>Befolkning och sociala perspektiv</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H31" s="2" t="inlineStr">
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ23J</t>
         </is>
@@ -1768,22 +1808,23 @@
           <t>2018-06-14</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr">
         <is>
           <t>Samhällsbyggnadsteknik</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
+      <c r="G32" t="inlineStr">
         <is>
           <t>Planeringsprojekt</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H32" s="2" t="inlineStr">
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ23K</t>
         </is>
@@ -1810,22 +1851,23 @@
           <t>2018-10-29</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr">
         <is>
           <t>Samhällsbyggnadsteknik</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="G33" t="inlineStr">
         <is>
           <t>Vetenskaplig metod</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H33" s="2" t="inlineStr">
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25J</t>
         </is>
@@ -1852,22 +1894,23 @@
           <t>2018-11-08</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr">
         <is>
           <t>Samhällsbyggnadsteknik</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
+      <c r="G34" t="inlineStr">
         <is>
           <t>Stadsbyggnad</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H34" s="2" t="inlineStr">
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25K</t>
         </is>
@@ -1894,22 +1937,23 @@
           <t>2019-01-31</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr">
         <is>
           <t>Maskinteknik</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr">
+      <c r="G35" t="inlineStr">
         <is>
           <t>Examensarbete Högskoleingenjör Maskinteknik</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H35" s="2" t="inlineStr">
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT25Z</t>
         </is>
@@ -1936,22 +1980,23 @@
           <t>2019-01-31</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr">
         <is>
           <t>Energiteknik</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
+      <c r="G36" t="inlineStr">
         <is>
           <t>Tillämpad solenergiteknik</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H36" s="2" t="inlineStr">
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG22R</t>
         </is>
@@ -1978,22 +2023,23 @@
           <t>2019-02-21</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr">
         <is>
           <t>Industriell ekonomi</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
+      <c r="G37" t="inlineStr">
         <is>
           <t>Industriell ekonomi - grundläggande kurs</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H37" s="2" t="inlineStr">
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE26P</t>
         </is>
@@ -2020,22 +2066,23 @@
           <t>2019-02-21</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr">
         <is>
           <t>Informatik</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
+      <c r="G38" t="inlineStr">
         <is>
           <t>Objektorienterad programmering och problemlösning</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H38" s="2" t="inlineStr">
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK289</t>
         </is>
@@ -2062,22 +2109,23 @@
           <t>2019-02-21</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr">
         <is>
           <t>Energiteknik</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
+      <c r="G39" t="inlineStr">
         <is>
           <t>Vetenskaplig kommunikation</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H39" s="2" t="inlineStr">
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG26J</t>
         </is>
@@ -2104,22 +2152,23 @@
           <t>2019-06-05</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr">
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr">
         <is>
           <t>Energiteknik</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr">
+      <c r="G40" t="inlineStr">
         <is>
           <t>Solel</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H40" s="2" t="inlineStr">
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG233</t>
         </is>
@@ -2146,22 +2195,23 @@
           <t>2019-06-13</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
+      <c r="E41" t="inlineStr"/>
+      <c r="F41" t="inlineStr">
         <is>
           <t>Industriell ekonomi</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr">
+      <c r="G41" t="inlineStr">
         <is>
           <t>Industriell ekonomi - Processer och projektledning</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H41" s="2" t="inlineStr">
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE29N</t>
         </is>
@@ -2190,20 +2240,25 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
+          <t>2019-09-19</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
           <t>Matematikdidaktik</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr">
+      <c r="G42" t="inlineStr">
         <is>
           <t>Matematikdidaktik I</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H42" s="2" t="inlineStr">
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2BH</t>
         </is>
@@ -2230,22 +2285,23 @@
           <t>2019-10-17</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
+      <c r="E43" t="inlineStr"/>
+      <c r="F43" t="inlineStr">
         <is>
           <t>Energiteknik</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr">
+      <c r="G43" t="inlineStr">
         <is>
           <t>Grundläggande forskningsmetodik</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H43" s="2" t="inlineStr">
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BEG222</t>
         </is>
@@ -2272,22 +2328,23 @@
           <t>2020-02-06</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr">
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr">
         <is>
           <t>Samhällsbyggnadsteknik</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr">
+      <c r="G44" t="inlineStr">
         <is>
           <t>Introduktion till GIS</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H44" s="2" t="inlineStr">
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2DH</t>
         </is>
@@ -2296,12 +2353,12 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>GMD2GF</t>
+          <t>GSQ2H7</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>SQQ</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2311,34 +2368,35 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>2020-04-08</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>Matematikdidaktik</t>
-        </is>
-      </c>
+          <t>2020-06-29</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr"/>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Matematik för lärare i åk 1-3, 30 hp (1-30). Ingår i Lärarlyftet.</t>
+          <t>Samhällsbyggnadsteknik</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H45" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2GF</t>
+          <t>Gestaltad livsmiljö</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2H7</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>GMD2H3</t>
+          <t>GMD2GF</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2353,39 +2411,44 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>2020-06-08</t>
+          <t>2020-04-08</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
+          <t>2020-12-15</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
           <t>Matematikdidaktik</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>Statistik och sannolikhetslära</t>
-        </is>
-      </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H46" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2H3</t>
+          <t>Matematik för lärare i åk 1-3, 30 hp (1-30). Ingår i Lärarlyftet.</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2GF</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>GMD2H5</t>
+          <t>GSQ2L9</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>SQQ</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2395,39 +2458,40 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>2020-06-08</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>Matematikdidaktik</t>
-        </is>
-      </c>
+          <t>2020-12-17</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Envariabelanalys</t>
+          <t>Samhällsbyggnadsteknik</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H47" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2H5</t>
+          <t>Geografiska Informationssystem för samhällsplanering</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I47" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2L9</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>GSQ2H7</t>
+          <t>GIE2MF</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>SQQ</t>
+          <t>IEA</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2437,39 +2501,40 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>2020-06-29</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>Samhällsbyggnadsteknik</t>
-        </is>
-      </c>
+          <t>2021-02-18</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr"/>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Gestaltad livsmiljö</t>
+          <t>Industriell ekonomi</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H48" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2H7</t>
+          <t>Industriell ekonomi - verksamhetsstyrning</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE2MF</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>GSQ2L9</t>
+          <t>GIK2PD</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>SQQ</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2479,39 +2544,40 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>2020-12-17</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>Samhällsbyggnadsteknik</t>
-        </is>
-      </c>
+          <t>2021-04-15</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr"/>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Geografiska Informationssystem för samhällsplanering</t>
+          <t>Informatik</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H49" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2L9</t>
+          <t>Hård infrastruktur</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2PD</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>GIE2MF</t>
+          <t>GMT2QF</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>IEA</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2521,34 +2587,35 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>2021-02-18</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>Industriell ekonomi</t>
-        </is>
-      </c>
+          <t>2021-05-20</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr"/>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Industriell ekonomi - verksamhetsstyrning</t>
+          <t>Maskinteknik</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H50" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE2MF</t>
+          <t>Finita element metoden i praktiken</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT2QF</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>GIK2PD</t>
+          <t>GIK2V4</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2563,39 +2630,40 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>2021-04-15</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
+          <t>2022-03-01</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr"/>
+      <c r="F51" t="inlineStr">
         <is>
           <t>Informatik</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>Hård infrastruktur</t>
-        </is>
-      </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H51" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2PD</t>
+          <t>Datasäkerhet och integritet</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2V4</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>GMT2QF</t>
+          <t>GEG2UL</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2605,39 +2673,40 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>2021-05-20</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>Maskinteknik</t>
-        </is>
-      </c>
+          <t>2022-03-01</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Finita element metoden i praktiken</t>
+          <t>Energiteknik</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H52" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT2QF</t>
+          <t>Förnybar kraftgenerering</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG2UL</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>GIK2V4</t>
+          <t>GMT2WL</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2647,39 +2716,40 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>2022-03-01</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>Informatik</t>
-        </is>
-      </c>
+          <t>2022-06-08</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr"/>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Datasäkerhet och integritet</t>
+          <t>Maskinteknik</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H53" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2V4</t>
+          <t>3D-printing översiktskurs</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I53" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT2WL</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>GEG2UL</t>
+          <t>GMD2XQ</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2689,39 +2759,40 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>2022-03-01</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>Energiteknik</t>
-        </is>
-      </c>
+          <t>2022-09-08</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Förnybar kraftgenerering</t>
+          <t>Matematikdidaktik</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H54" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG2UL</t>
+          <t>Matematik för lärare i gymnasieskolan, 90 hp (1-90 hp). Ingår i lärarlyftet</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2XQ</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>GMT2WL</t>
+          <t>GIK2YK</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2731,39 +2802,40 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>2022-06-08</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>Maskinteknik</t>
-        </is>
-      </c>
+          <t>2022-11-29</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr">
         <is>
-          <t>3D-printing översiktskurs</t>
+          <t>Informatik</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H55" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT2WL</t>
+          <t>Relationsdatabaser</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I55" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2YK</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>GMD2XQ</t>
+          <t>GIK2YL</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2773,34 +2845,35 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>2022-09-08</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>Matematikdidaktik</t>
-        </is>
-      </c>
+          <t>2022-11-29</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Matematik för lärare i gymnasieskolan, 90 hp (1-90 hp). Ingår i lärarlyftet</t>
+          <t>Informatik</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H56" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2XQ</t>
+          <t>Projekt och agila arbetsmetoder</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2YL</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>GIK2YK</t>
+          <t>GIK2YN</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2818,31 +2891,32 @@
           <t>2022-11-29</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr">
+      <c r="E57" t="inlineStr"/>
+      <c r="F57" t="inlineStr">
         <is>
           <t>Informatik</t>
         </is>
       </c>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t>Relationsdatabaser</t>
-        </is>
-      </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H57" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2YK</t>
+          <t>Programutvecklingsteknik</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I57" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2YN</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>GIK2YL</t>
+          <t>GIK2YP</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2860,31 +2934,32 @@
           <t>2022-11-29</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr">
+      <c r="E58" t="inlineStr"/>
+      <c r="F58" t="inlineStr">
         <is>
           <t>Informatik</t>
         </is>
       </c>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>Projekt och agila arbetsmetoder</t>
-        </is>
-      </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H58" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2YL</t>
+          <t>Webbdesign</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2YP</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>GIK2YN</t>
+          <t>GIK2YR</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2902,36 +2977,37 @@
           <t>2022-11-29</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr">
+      <c r="E59" t="inlineStr"/>
+      <c r="F59" t="inlineStr">
         <is>
           <t>Informatik</t>
         </is>
       </c>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>Programutvecklingsteknik</t>
-        </is>
-      </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H59" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2YN</t>
+          <t>Designprinciper och användargränssnitt</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I59" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2YR</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>GIK2YP</t>
+          <t>GEG2ZQ</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2941,34 +3017,35 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>2022-11-29</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>Informatik</t>
-        </is>
-      </c>
+          <t>2022-12-20</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr"/>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Webbdesign</t>
+          <t>Energiteknik</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H60" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2YP</t>
+          <t>Solenergi</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I60" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG2ZQ</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>GIK2YR</t>
+          <t>GIK32K</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2983,34 +3060,35 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>2022-11-29</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
+          <t>2023-02-07</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr"/>
+      <c r="F61" t="inlineStr">
         <is>
           <t>Informatik</t>
         </is>
       </c>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>Designprinciper och användargränssnitt</t>
-        </is>
-      </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H61" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2YR</t>
+          <t>Layout och typografi</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I61" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK32K</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>GEG2ZQ</t>
+          <t>GEG33A</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -3025,39 +3103,40 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>2022-12-20</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
+          <t>2023-02-23</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr"/>
+      <c r="F62" t="inlineStr">
         <is>
           <t>Energiteknik</t>
         </is>
       </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>Solenergi</t>
-        </is>
-      </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H62" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG2ZQ</t>
+          <t>Installation av solcellssystem</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I62" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG33A</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>GIK32K</t>
+          <t>GMD33X</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -3067,39 +3146,40 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>2023-02-07</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>Informatik</t>
-        </is>
-      </c>
+          <t>2023-03-17</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Layout och typografi</t>
+          <t>Matematikdidaktik</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H63" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK32K</t>
+          <t>Matematik för lärare i åk 7-9</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I63" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD33X</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>GEG33A</t>
+          <t>GMD33Y</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -3109,39 +3189,40 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>2023-02-23</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>Energiteknik</t>
-        </is>
-      </c>
+          <t>2023-03-17</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr"/>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Installation av solcellssystem</t>
+          <t>Matematikdidaktik</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H64" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG33A</t>
+          <t>Matematik för lärare i gymnasieskolan</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I64" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD33Y</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>GMD33X</t>
+          <t>GBY34B</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>BYA</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -3151,39 +3232,40 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>2023-03-17</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>Matematikdidaktik</t>
-        </is>
-      </c>
+          <t>2023-04-04</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Matematik för lärare i åk 7-9</t>
+          <t>Byggteknik</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H65" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD33X</t>
+          <t>Vägplanering</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY34B</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>GMD33Y</t>
+          <t>GIK346</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -3193,39 +3275,40 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>2023-03-17</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>Matematikdidaktik</t>
-        </is>
-      </c>
+          <t>2023-04-04</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Matematik för lärare i gymnasieskolan</t>
+          <t>Informatik</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H66" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD33Y</t>
+          <t>Data Science programmering och dataanalys</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I66" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK346</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>GBY34B</t>
+          <t>GMD2H3</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>BYA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -3235,39 +3318,44 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>2023-04-04</t>
+          <t>2020-06-08</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Byggteknik</t>
+          <t>2023-04-21</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Vägplanering</t>
+          <t>Matematikdidaktik</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H67" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY34B</t>
+          <t>Statistik och sannolikhetslära</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I67" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2H3</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>GIK346</t>
+          <t>GMD2H5</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -3277,27 +3365,32 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>2023-04-04</t>
+          <t>2020-06-08</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Informatik</t>
+          <t>2023-04-21</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Data Science programmering och dataanalys</t>
+          <t>Matematikdidaktik</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H68" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK346</t>
+          <t>Envariabelanalys</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I68" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2H5</t>
         </is>
       </c>
     </row>
@@ -3322,22 +3415,23 @@
           <t>2023-10-31</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr">
+      <c r="E69" t="inlineStr"/>
+      <c r="F69" t="inlineStr">
         <is>
           <t>Informatik</t>
         </is>
       </c>
-      <c r="F69" t="inlineStr">
+      <c r="G69" t="inlineStr">
         <is>
           <t>Komponentdriven webbdesign</t>
         </is>
       </c>
-      <c r="G69" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H69" s="2" t="inlineStr">
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I69" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK375</t>
         </is>
@@ -3364,22 +3458,23 @@
           <t>2023-10-31</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr">
+      <c r="E70" t="inlineStr"/>
+      <c r="F70" t="inlineStr">
         <is>
           <t>Informatik</t>
         </is>
       </c>
-      <c r="F70" t="inlineStr">
+      <c r="G70" t="inlineStr">
         <is>
           <t>Applikationsutveckling för webben</t>
         </is>
       </c>
-      <c r="G70" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H70" s="2" t="inlineStr">
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I70" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK376</t>
         </is>
@@ -3406,22 +3501,23 @@
           <t>2023-12-19</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr">
+      <c r="E71" t="inlineStr"/>
+      <c r="F71" t="inlineStr">
         <is>
           <t>Informatik</t>
         </is>
       </c>
-      <c r="F71" t="inlineStr">
+      <c r="G71" t="inlineStr">
         <is>
           <t>Design av digitala tjänster</t>
         </is>
       </c>
-      <c r="G71" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H71" s="2" t="inlineStr">
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I71" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK38G</t>
         </is>
@@ -3448,22 +3544,23 @@
           <t>2023-12-19</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr">
+      <c r="E72" t="inlineStr"/>
+      <c r="F72" t="inlineStr">
         <is>
           <t>Informatik</t>
         </is>
       </c>
-      <c r="F72" t="inlineStr">
+      <c r="G72" t="inlineStr">
         <is>
           <t>Introduktion till IT och digitala tjänster</t>
         </is>
       </c>
-      <c r="G72" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H72" s="2" t="inlineStr">
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I72" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK38H</t>
         </is>
@@ -3490,22 +3587,23 @@
           <t>2024-05-23</t>
         </is>
       </c>
-      <c r="E73" t="inlineStr">
+      <c r="E73" t="inlineStr"/>
+      <c r="F73" t="inlineStr">
         <is>
           <t>Informatik</t>
         </is>
       </c>
-      <c r="F73" t="inlineStr">
+      <c r="G73" t="inlineStr">
         <is>
           <t>E-samhället: e-förvaltning och digitala tjänster</t>
         </is>
       </c>
-      <c r="G73" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H73" s="2" t="inlineStr">
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I73" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK3BV</t>
         </is>
@@ -3532,22 +3630,23 @@
           <t>2024-06-13</t>
         </is>
       </c>
-      <c r="E74" t="inlineStr">
+      <c r="E74" t="inlineStr"/>
+      <c r="F74" t="inlineStr">
         <is>
           <t>Energiteknik</t>
         </is>
       </c>
-      <c r="F74" t="inlineStr">
+      <c r="G74" t="inlineStr">
         <is>
           <t>Elektriska lagringssystem och tjänster</t>
         </is>
       </c>
-      <c r="G74" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H74" s="2" t="inlineStr">
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I74" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2AY</t>
         </is>
@@ -3574,22 +3673,23 @@
           <t>2024-06-13</t>
         </is>
       </c>
-      <c r="E75" t="inlineStr">
+      <c r="E75" t="inlineStr"/>
+      <c r="F75" t="inlineStr">
         <is>
           <t>Energiteknik</t>
         </is>
       </c>
-      <c r="F75" t="inlineStr">
+      <c r="G75" t="inlineStr">
         <is>
           <t>Projektkurs 3 - grupprojekt och kommunikation</t>
         </is>
       </c>
-      <c r="G75" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H75" s="2" t="inlineStr">
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I75" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2B5</t>
         </is>
@@ -3616,22 +3716,23 @@
           <t>2024-12-12</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr">
+      <c r="E76" t="inlineStr"/>
+      <c r="F76" t="inlineStr">
         <is>
           <t>Energiteknik</t>
         </is>
       </c>
-      <c r="F76" t="inlineStr">
+      <c r="G76" t="inlineStr">
         <is>
           <t>Hållbarhet hos solenergisystem</t>
         </is>
       </c>
-      <c r="G76" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H76" s="2" t="inlineStr">
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I76" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2AV</t>
         </is>
@@ -3658,22 +3759,23 @@
           <t>2024-12-12</t>
         </is>
       </c>
-      <c r="E77" t="inlineStr">
+      <c r="E77" t="inlineStr"/>
+      <c r="F77" t="inlineStr">
         <is>
           <t>Energiteknik</t>
         </is>
       </c>
-      <c r="F77" t="inlineStr">
+      <c r="G77" t="inlineStr">
         <is>
           <t>Urbana energisystem</t>
         </is>
       </c>
-      <c r="G77" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H77" s="2" t="inlineStr">
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I77" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2AW</t>
         </is>
@@ -3700,22 +3802,23 @@
           <t>2024-12-12</t>
         </is>
       </c>
-      <c r="E78" t="inlineStr">
+      <c r="E78" t="inlineStr"/>
+      <c r="F78" t="inlineStr">
         <is>
           <t>Energiteknik</t>
         </is>
       </c>
-      <c r="F78" t="inlineStr">
+      <c r="G78" t="inlineStr">
         <is>
           <t>Elnätsintegrering av förnybar kraft</t>
         </is>
       </c>
-      <c r="G78" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H78" s="2" t="inlineStr">
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I78" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2AX</t>
         </is>
@@ -3742,22 +3845,23 @@
           <t>2025-05-22</t>
         </is>
       </c>
-      <c r="E79" t="inlineStr">
+      <c r="E79" t="inlineStr"/>
+      <c r="F79" t="inlineStr">
         <is>
           <t>Matematikdidaktik</t>
         </is>
       </c>
-      <c r="F79" t="inlineStr">
+      <c r="G79" t="inlineStr">
         <is>
           <t>Matematikutveckling i förskoleklass och årskurs 1–3 utifrån första- och andraspråksperspektiv</t>
         </is>
       </c>
-      <c r="G79" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H79" s="2" t="inlineStr">
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I79" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD3FX</t>
         </is>
@@ -3784,22 +3888,23 @@
           <t>2025-05-22</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr">
+      <c r="E80" t="inlineStr"/>
+      <c r="F80" t="inlineStr">
         <is>
           <t>Energiteknik</t>
         </is>
       </c>
-      <c r="F80" t="inlineStr">
+      <c r="G80" t="inlineStr">
         <is>
           <t>Praktik inom energiteknik</t>
         </is>
       </c>
-      <c r="G80" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H80" s="2" t="inlineStr">
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I80" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG3FY</t>
         </is>
@@ -3826,22 +3931,23 @@
           <t>2026-03-30</t>
         </is>
       </c>
-      <c r="E81" t="inlineStr">
+      <c r="E81" t="inlineStr"/>
+      <c r="F81" t="inlineStr">
         <is>
           <t>Maskinteknik</t>
         </is>
       </c>
-      <c r="F81" t="inlineStr">
+      <c r="G81" t="inlineStr">
         <is>
           <t>Mekatronik</t>
         </is>
       </c>
-      <c r="G81" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H81" s="2" t="inlineStr">
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I81" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3JQ</t>
         </is>
@@ -3868,22 +3974,23 @@
           <t>2026-03-30</t>
         </is>
       </c>
-      <c r="E82" t="inlineStr">
+      <c r="E82" t="inlineStr"/>
+      <c r="F82" t="inlineStr">
         <is>
           <t>Maskinteknik</t>
         </is>
       </c>
-      <c r="F82" t="inlineStr">
+      <c r="G82" t="inlineStr">
         <is>
           <t>Termodynamik</t>
         </is>
       </c>
-      <c r="G82" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H82" s="2" t="inlineStr">
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I82" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3JR</t>
         </is>
@@ -3910,22 +4017,23 @@
           <t>2026-03-30</t>
         </is>
       </c>
-      <c r="E83" t="inlineStr">
+      <c r="E83" t="inlineStr"/>
+      <c r="F83" t="inlineStr">
         <is>
           <t>Maskinteknik</t>
         </is>
       </c>
-      <c r="F83" t="inlineStr">
+      <c r="G83" t="inlineStr">
         <is>
           <t>Tillverkning</t>
         </is>
       </c>
-      <c r="G83" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H83" s="2" t="inlineStr">
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I83" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3JY</t>
         </is>
@@ -3952,22 +4060,23 @@
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="E84" t="inlineStr">
+      <c r="E84" t="inlineStr"/>
+      <c r="F84" t="inlineStr">
         <is>
           <t>Industriell ekonomi</t>
         </is>
       </c>
-      <c r="F84" t="inlineStr">
+      <c r="G84" t="inlineStr">
         <is>
           <t>Innovation och entreprenörskap inom assisterande teknik</t>
         </is>
       </c>
-      <c r="G84" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H84" s="2" t="inlineStr">
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I84" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE3JW</t>
         </is>
@@ -3994,22 +4103,23 @@
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="E85" t="inlineStr">
+      <c r="E85" t="inlineStr"/>
+      <c r="F85" t="inlineStr">
         <is>
           <t>Maskinteknik</t>
         </is>
       </c>
-      <c r="F85" t="inlineStr">
+      <c r="G85" t="inlineStr">
         <is>
           <t>Tillämpning av regelverk för assisterande produkter</t>
         </is>
       </c>
-      <c r="G85" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H85" s="2" t="inlineStr">
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I85" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3JT</t>
         </is>
@@ -4036,22 +4146,23 @@
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr">
+      <c r="E86" t="inlineStr"/>
+      <c r="F86" t="inlineStr">
         <is>
           <t>Maskinteknik</t>
         </is>
       </c>
-      <c r="F86" t="inlineStr">
+      <c r="G86" t="inlineStr">
         <is>
           <t>Smarta hem och e-hälsoteknik</t>
         </is>
       </c>
-      <c r="G86" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H86" s="2" t="inlineStr">
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I86" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3JU</t>
         </is>
@@ -4078,202 +4189,203 @@
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr">
+      <c r="E87" t="inlineStr"/>
+      <c r="F87" t="inlineStr">
         <is>
           <t>Maskinteknik</t>
         </is>
       </c>
-      <c r="F87" t="inlineStr">
+      <c r="G87" t="inlineStr">
         <is>
           <t>Assisterande robotik</t>
         </is>
       </c>
-      <c r="G87" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång hittad på kurssidan</t>
-        </is>
-      </c>
-      <c r="H87" s="2" t="inlineStr">
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I87" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3JV</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H87"/>
+  <autoFilter ref="A1:I87"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I2" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I3" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I4" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A6" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A7" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A8" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A9" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A10" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A11" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A12" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I12" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A13" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I13" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A14" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="rId26"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A15" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="rId28"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A16" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I16" r:id="rId30"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A17" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId32"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A18" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="rId34"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A19" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="rId36"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A20" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="rId38"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A21" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="rId40"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A22" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="rId42"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A23" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="rId44"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A24" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="rId46"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A25" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="rId48"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A26" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="rId50"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A27" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId52"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A28" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="rId54"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A29" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I29" r:id="rId56"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A30" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H30" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I30" r:id="rId58"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A31" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H31" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I31" r:id="rId60"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A32" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H32" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I32" r:id="rId62"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A33" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H33" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I33" r:id="rId64"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A34" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I34" r:id="rId66"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A35" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H35" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="rId68"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A36" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H36" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I36" r:id="rId70"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A37" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H37" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="rId72"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A38" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H38" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I38" r:id="rId74"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A39" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H39" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I39" r:id="rId76"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A40" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H40" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="rId78"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A41" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H41" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I41" r:id="rId80"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A42" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H42" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I42" r:id="rId82"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A43" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H43" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I43" r:id="rId84"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A44" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H44" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I44" r:id="rId86"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A45" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H45" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I45" r:id="rId88"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A46" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H46" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I46" r:id="rId90"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A47" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H47" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I47" r:id="rId92"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A48" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H48" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I48" r:id="rId94"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A49" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H49" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I49" r:id="rId96"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A50" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H50" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I50" r:id="rId98"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A51" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H51" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I51" r:id="rId100"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A52" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H52" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I52" r:id="rId102"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A53" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H53" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I53" r:id="rId104"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A54" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H54" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I54" r:id="rId106"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A55" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H55" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I55" r:id="rId108"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A56" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H56" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I56" r:id="rId110"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A57" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H57" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I57" r:id="rId112"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A58" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H58" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I58" r:id="rId114"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A59" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H59" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I59" r:id="rId116"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A60" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H60" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I60" r:id="rId118"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A61" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H61" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I61" r:id="rId120"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A62" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H62" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I62" r:id="rId122"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A63" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H63" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I63" r:id="rId124"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A64" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H64" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I64" r:id="rId126"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A65" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H65" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I65" r:id="rId128"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A66" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H66" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I66" r:id="rId130"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A67" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H67" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I67" r:id="rId132"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A68" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H68" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I68" r:id="rId134"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A69" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H69" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I69" r:id="rId136"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A70" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H70" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I70" r:id="rId138"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A71" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H71" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I71" r:id="rId140"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A72" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H72" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I72" r:id="rId142"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A73" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H73" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I73" r:id="rId144"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A74" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H74" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I74" r:id="rId146"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A75" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H75" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I75" r:id="rId148"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A76" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H76" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I76" r:id="rId150"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A77" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H77" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I77" r:id="rId152"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A78" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H78" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I78" r:id="rId154"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A79" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H79" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I79" r:id="rId156"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A80" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H80" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I80" r:id="rId158"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A81" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H81" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I81" r:id="rId160"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A82" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H82" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I82" r:id="rId162"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A83" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H83" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I83" r:id="rId164"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A84" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H84" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I84" r:id="rId166"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A85" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H85" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I85" r:id="rId168"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A86" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H86" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I86" r:id="rId170"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A87" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H87" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I87" r:id="rId172"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update course codes and course plan documents for various programs; add new course materials for postgraduate studies in Pedagogical Work.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/01 IIT/Analys/Vilande kursplaner.xlsx
+++ b/vault-dalarna-university/01 IIT/Analys/Vilande kursplaner.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Vilande kursplaner" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Vilande kursplaner'!$A$1:$I$88</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Vilande kursplaner'!$A$1:$I$101</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I88"/>
+  <dimension ref="A1:I101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -625,12 +625,12 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>BY2016</t>
+          <t>MIKR002</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>BYA</t>
+          <t>MIKRODAT</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -640,18 +640,18 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2013-02-21</t>
+          <t>2012-12-04</t>
         </is>
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Byggteknik</t>
+          <t>Mikrodataanalys</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Examensarbete i byggteknik för högskoleingenjörsexamen</t>
+          <t>Datainsamling och datakvalitet</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -661,14 +661,14 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY2016</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MIKR002</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>BY1047</t>
+          <t>BY2016</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -683,7 +683,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2013-03-14</t>
+          <t>2013-02-21</t>
         </is>
       </c>
       <c r="E6" t="inlineStr"/>
@@ -694,7 +694,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Bärkraftigt byggande och boende</t>
+          <t>Examensarbete i byggteknik för högskoleingenjörsexamen</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -704,19 +704,19 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY1047</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY2016</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>IK1066</t>
+          <t>BY1047</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>BYA</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -732,12 +732,12 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Informatik</t>
+          <t>Byggteknik</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Förändringsanalys</t>
+          <t>Bärkraftigt byggande och boende</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -747,19 +747,19 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IK1066</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY1047</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>MD1085</t>
+          <t>IK1066</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -769,18 +769,18 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2013-12-17</t>
+          <t>2013-03-14</t>
         </is>
       </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Matematikdidaktik</t>
+          <t>Informatik</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Matematikundervisning i ett specialpedagogiskt perspektiv</t>
+          <t>Förändringsanalys</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -790,19 +790,19 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD1085</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IK1066</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>MT1060</t>
+          <t>MD1085</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -812,18 +812,18 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2014-04-03</t>
+          <t>2013-12-17</t>
         </is>
       </c>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Maskinteknik</t>
+          <t>Matematikdidaktik</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Hållfasthetslära</t>
+          <t>Matematikundervisning i ett specialpedagogiskt perspektiv</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -833,19 +833,19 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1060</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD1085</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>IK1064</t>
+          <t>MT1060</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -855,22 +855,18 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2013-02-21</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>2014-09-01</t>
-        </is>
-      </c>
+          <t>2014-04-03</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Informatik</t>
+          <t>Maskinteknik</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Datahantering och Problemlösning</t>
+          <t>Hållfasthetslära</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -880,19 +876,19 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IK1064</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1060</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>EG4001</t>
+          <t>IK1064</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -902,18 +898,22 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2014-11-27</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr"/>
+          <t>2013-02-21</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>2014-09-01</t>
+        </is>
+      </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Energiteknik</t>
+          <t>Informatik</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Examensarbete för masterexamen i solenergiteknik</t>
+          <t>Datahantering och Problemlösning</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -923,19 +923,19 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG4001</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IK1064</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>MD1097</t>
+          <t>MÖ4005</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -945,18 +945,22 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2015-03-05</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr"/>
+          <t>2014-01-30</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>2014-10-09</t>
+        </is>
+      </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Matematikdidaktik</t>
+          <t>Energiteknik</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Matematikens historia för lärare</t>
+          <t>Projektkurs i solenergisystem eller energieffektiva byggnader</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -966,19 +970,19 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD1097</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MÖ4005</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>MD1098</t>
+          <t>EG4001</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -988,18 +992,18 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2015-03-05</t>
+          <t>2014-11-27</t>
         </is>
       </c>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Matematikdidaktik</t>
+          <t>Energiteknik</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Matematisk problemlösning i grundskolans senare år</t>
+          <t>Examensarbete för masterexamen i solenergiteknik</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1009,19 +1013,19 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD1098</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG4001</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>BY1059</t>
+          <t>MD1097</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>BYA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1031,18 +1035,18 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2015-03-20</t>
+          <t>2015-03-05</t>
         </is>
       </c>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Byggteknik</t>
+          <t>Matematikdidaktik</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Praktisk byggteknik</t>
+          <t>Matematikens historia för lärare</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1052,19 +1056,19 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY1059</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD1097</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>EG3007</t>
+          <t>MD1098</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1074,18 +1078,18 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2015-08-27</t>
+          <t>2015-03-05</t>
         </is>
       </c>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Energiteknik</t>
+          <t>Matematikdidaktik</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Solvärme</t>
+          <t>Matematisk problemlösning i grundskolans senare år</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1095,19 +1099,19 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3007</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD1098</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>EG3015</t>
+          <t>BY1059</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>BYA</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1117,18 +1121,18 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2015-08-27</t>
+          <t>2015-03-20</t>
         </is>
       </c>
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Energiteknik</t>
+          <t>Byggteknik</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Solstrålning och solgeometri</t>
+          <t>Praktisk byggteknik</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1138,14 +1142,14 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3015</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY1059</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>EG3012</t>
+          <t>EG3007</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1160,7 +1164,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2015-09-17</t>
+          <t>2015-08-27</t>
         </is>
       </c>
       <c r="E17" t="inlineStr"/>
@@ -1171,7 +1175,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Hållbara energisystem</t>
+          <t>Solvärme</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1181,19 +1185,19 @@
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3012</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3007</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>BY1061</t>
+          <t>EG3015</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>BYA</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1203,18 +1207,18 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2015-11-23</t>
+          <t>2015-08-27</t>
         </is>
       </c>
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Byggteknik</t>
+          <t>Energiteknik</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Installationsteknik och dimensionering</t>
+          <t>Solstrålning och solgeometri</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1224,19 +1228,19 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY1061</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3015</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>MA1040</t>
+          <t>EG3012</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>MAA</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1246,18 +1250,18 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2016-03-24</t>
+          <t>2015-09-17</t>
         </is>
       </c>
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Matematik</t>
+          <t>Energiteknik</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Matematik för tekniker</t>
+          <t>Hållbara energisystem</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1267,14 +1271,14 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MA1040</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3012</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>BY2022</t>
+          <t>BY1061</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1289,7 +1293,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2016-05-19</t>
+          <t>2015-11-23</t>
         </is>
       </c>
       <c r="E20" t="inlineStr"/>
@@ -1300,7 +1304,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Energiprojekt</t>
+          <t>Installationsteknik och dimensionering</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1310,19 +1314,19 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY2022</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY1061</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>MT1068</t>
+          <t>MA1040</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>MAA</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1332,18 +1336,18 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2016-05-19</t>
+          <t>2016-03-24</t>
         </is>
       </c>
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Maskinteknik</t>
+          <t>Matematik</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Introduktion till produktutveckling</t>
+          <t>Matematik för tekniker</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1353,14 +1357,14 @@
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1068</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MA1040</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>BY1065</t>
+          <t>BY2022</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1375,7 +1379,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2016-09-01</t>
+          <t>2016-05-19</t>
         </is>
       </c>
       <c r="E22" t="inlineStr"/>
@@ -1386,7 +1390,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>BIM projekt och projektering</t>
+          <t>Energiprojekt</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1396,19 +1400,19 @@
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY1065</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY2022</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>EG3017</t>
+          <t>MT1068</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1418,18 +1422,18 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2016-09-22</t>
+          <t>2016-05-19</t>
         </is>
       </c>
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Energiteknik</t>
+          <t>Maskinteknik</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Solenergiteknikpraktik</t>
+          <t>Introduktion till produktutveckling</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1439,19 +1443,19 @@
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3017</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1068</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>EG3018</t>
+          <t>BY1065</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>BYA</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1461,18 +1465,18 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2016-09-22</t>
+          <t>2016-09-01</t>
         </is>
       </c>
       <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Energiteknik</t>
+          <t>Byggteknik</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Solenergiteknikpraktik</t>
+          <t>BIM projekt och projektering</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -1482,19 +1486,19 @@
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3018</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY1065</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>MA1042</t>
+          <t>EG3017</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>MAA</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1504,18 +1508,18 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2017-02-16</t>
+          <t>2016-09-22</t>
         </is>
       </c>
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Matematik</t>
+          <t>Energiteknik</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Flervariabelanalys</t>
+          <t>Solenergiteknikpraktik</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1525,19 +1529,19 @@
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MA1042</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3017</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>SQ1003</t>
+          <t>EG3018</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>SQQ</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1547,18 +1551,18 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2017-10-12</t>
+          <t>2016-09-22</t>
         </is>
       </c>
       <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Samhällsbyggnadsteknik</t>
+          <t>Energiteknik</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Vetenskapligt metod</t>
+          <t>Solenergiteknikpraktik</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -1568,19 +1572,19 @@
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SQ1003</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3018</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>BY3005</t>
+          <t>MA1042</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>BYA</t>
+          <t>MAA</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1590,18 +1594,18 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>2017-12-14</t>
+          <t>2017-02-16</t>
         </is>
       </c>
       <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Byggteknik</t>
+          <t>Matematik</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Hållbar samhällsplanering</t>
+          <t>Flervariabelanalys</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -1611,19 +1615,19 @@
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY3005</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MA1042</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>MT1074</t>
+          <t>FMI2223</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>MIKRODAT</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1633,18 +1637,18 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>2018-02-15</t>
+          <t>2017-10-04</t>
         </is>
       </c>
       <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Maskinteknik</t>
+          <t>Mikrodataanalys</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Maskinelement</t>
+          <t>Komplexitet och operationsanalytiska metoder för forskarstuderande</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -1654,19 +1658,19 @@
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1074</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FMI2223</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>GMT228</t>
+          <t>SQ1003</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>SQQ</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1676,18 +1680,18 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>2018-04-05</t>
+          <t>2017-10-12</t>
         </is>
       </c>
       <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Maskinteknik</t>
+          <t>Samhällsbyggnadsteknik</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Produktutvecklingsmetoder</t>
+          <t>Vetenskapligt metod</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -1697,19 +1701,19 @@
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT228</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SQ1003</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>AEG225</t>
+          <t>BY3005</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>BYA</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1719,18 +1723,18 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>2018-05-24</t>
+          <t>2017-12-14</t>
         </is>
       </c>
       <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Energiteknik</t>
+          <t>Byggteknik</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Solenergins ekonomi</t>
+          <t>Hållbar samhällsplanering</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -1740,19 +1744,19 @@
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG225</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY3005</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>GSQ23J</t>
+          <t>MT1074</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>SQQ</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1762,18 +1766,18 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>2018-05-24</t>
+          <t>2018-02-15</t>
         </is>
       </c>
       <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Samhällsbyggnadsteknik</t>
+          <t>Maskinteknik</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Befolkning och sociala perspektiv</t>
+          <t>Maskinelement</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -1783,19 +1787,19 @@
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ23J</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1074</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>GSQ23K</t>
+          <t>GMT228</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>SQQ</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1805,18 +1809,18 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>2018-06-14</t>
+          <t>2018-04-05</t>
         </is>
       </c>
       <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Samhällsbyggnadsteknik</t>
+          <t>Maskinteknik</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Planeringsprojekt</t>
+          <t>Produktutvecklingsmetoder</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -1826,19 +1830,19 @@
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ23K</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT228</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>GSQ25J</t>
+          <t>AEG225</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>SQQ</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1848,18 +1852,18 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>2018-10-29</t>
+          <t>2018-05-24</t>
         </is>
       </c>
       <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Samhällsbyggnadsteknik</t>
+          <t>Energiteknik</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Vetenskaplig metod</t>
+          <t>Solenergins ekonomi</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -1869,14 +1873,14 @@
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25J</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG225</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>GSQ25K</t>
+          <t>GSQ23J</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1891,7 +1895,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>2018-11-08</t>
+          <t>2018-05-24</t>
         </is>
       </c>
       <c r="E34" t="inlineStr"/>
@@ -1902,7 +1906,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Stadsbyggnad</t>
+          <t>Befolkning och sociala perspektiv</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -1912,19 +1916,19 @@
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25K</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ23J</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>GMT25Z</t>
+          <t>GSQ23K</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>SQQ</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1934,18 +1938,18 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>2019-01-31</t>
+          <t>2018-06-14</t>
         </is>
       </c>
       <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Maskinteknik</t>
+          <t>Samhällsbyggnadsteknik</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Examensarbete Högskoleingenjör Maskinteknik</t>
+          <t>Planeringsprojekt</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -1955,19 +1959,19 @@
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT25Z</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ23K</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>AEG22R</t>
+          <t>GSQ25J</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>SQQ</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1977,18 +1981,18 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>2019-01-31</t>
+          <t>2018-10-29</t>
         </is>
       </c>
       <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Energiteknik</t>
+          <t>Samhällsbyggnadsteknik</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Tillämpad solenergiteknik</t>
+          <t>Vetenskaplig metod</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -1998,19 +2002,19 @@
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG22R</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25J</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>GIE26P</t>
+          <t>GSQ25K</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>IEA</t>
+          <t>SQQ</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2020,18 +2024,18 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>2019-02-21</t>
+          <t>2018-11-08</t>
         </is>
       </c>
       <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Industriell ekonomi</t>
+          <t>Samhällsbyggnadsteknik</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Industriell ekonomi - grundläggande kurs</t>
+          <t>Stadsbyggnad</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -2041,19 +2045,19 @@
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE26P</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25K</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>GIK289</t>
+          <t>GMT25Z</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2063,18 +2067,18 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>2019-02-21</t>
+          <t>2019-01-31</t>
         </is>
       </c>
       <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Informatik</t>
+          <t>Maskinteknik</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Objektorienterad programmering och problemlösning</t>
+          <t>Examensarbete Högskoleingenjör Maskinteknik</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -2084,14 +2088,14 @@
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK289</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT25Z</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>GEG26J</t>
+          <t>AEG22R</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2106,7 +2110,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>2019-02-21</t>
+          <t>2019-01-31</t>
         </is>
       </c>
       <c r="E39" t="inlineStr"/>
@@ -2117,7 +2121,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Vetenskaplig kommunikation</t>
+          <t>Tillämpad solenergiteknik</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -2127,19 +2131,19 @@
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG26J</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG22R</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>AEG233</t>
+          <t>GIE26P</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>IEA</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2149,18 +2153,18 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>2019-06-05</t>
+          <t>2019-02-21</t>
         </is>
       </c>
       <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Energiteknik</t>
+          <t>Industriell ekonomi</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Solel</t>
+          <t>Industriell ekonomi - grundläggande kurs</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -2170,19 +2174,19 @@
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG233</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE26P</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>GIE29N</t>
+          <t>GIK289</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>IEA</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2192,18 +2196,18 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>2019-06-13</t>
+          <t>2019-02-21</t>
         </is>
       </c>
       <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Industriell ekonomi</t>
+          <t>Informatik</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Industriell ekonomi - Processer och projektledning</t>
+          <t>Objektorienterad programmering och problemlösning</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -2213,19 +2217,19 @@
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE29N</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK289</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>GMD2BH</t>
+          <t>GEG26J</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2235,22 +2239,18 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>2019-08-29</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>2019-09-19</t>
-        </is>
-      </c>
+          <t>2019-02-21</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Matematikdidaktik</t>
+          <t>Energiteknik</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Matematikdidaktik I</t>
+          <t>Vetenskaplig kommunikation</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -2260,14 +2260,14 @@
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2BH</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG26J</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>BEG222</t>
+          <t>AEG233</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2282,7 +2282,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>2019-10-17</t>
+          <t>2019-06-05</t>
         </is>
       </c>
       <c r="E43" t="inlineStr"/>
@@ -2293,7 +2293,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Grundläggande forskningsmetodik</t>
+          <t>Solel</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -2303,19 +2303,19 @@
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BEG222</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG233</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>GSQ2DH</t>
+          <t>GIE29N</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>SQQ</t>
+          <t>IEA</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2325,18 +2325,18 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>2020-02-06</t>
+          <t>2019-06-13</t>
         </is>
       </c>
       <c r="E44" t="inlineStr"/>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Samhällsbyggnadsteknik</t>
+          <t>Industriell ekonomi</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Introduktion till GIS</t>
+          <t>Industriell ekonomi - Processer och projektledning</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -2346,19 +2346,19 @@
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2DH</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE29N</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>GSQ2H7</t>
+          <t>GMD2BH</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>SQQ</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2368,18 +2368,22 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>2020-06-29</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr"/>
+          <t>2019-08-29</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>2019-09-19</t>
+        </is>
+      </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Samhällsbyggnadsteknik</t>
+          <t>Matematikdidaktik</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Gestaltad livsmiljö</t>
+          <t>Matematikdidaktik I</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -2389,19 +2393,19 @@
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2H7</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2BH</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>GMD2GF</t>
+          <t>FMI2222</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>MIKRODAT</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2411,22 +2415,18 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>2020-04-08</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>2020-12-15</t>
-        </is>
-      </c>
+          <t>2019-10-03</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Matematikdidaktik</t>
+          <t>Mikrodataanalys</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Matematik för lärare i åk 1-3, 30 hp (1-30). Ingår i Lärarlyftet.</t>
+          <t>Ledarskapets ekonomi för forskarstuderande</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -2436,19 +2436,19 @@
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2GF</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FMI2222</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>GSQ2L9</t>
+          <t>BEG222</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>SQQ</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2458,18 +2458,18 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>2020-12-17</t>
+          <t>2019-10-17</t>
         </is>
       </c>
       <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Samhällsbyggnadsteknik</t>
+          <t>Energiteknik</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Geografiska Informationssystem för samhällsplanering</t>
+          <t>Grundläggande forskningsmetodik</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -2479,19 +2479,19 @@
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2L9</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BEG222</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>GIE2MF</t>
+          <t>FMI2224</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>IEA</t>
+          <t>MIKRODAT</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2501,18 +2501,18 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>2021-02-18</t>
+          <t>2019-10-29</t>
         </is>
       </c>
       <c r="E48" t="inlineStr"/>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Industriell ekonomi</t>
+          <t>Mikrodataanalys</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Industriell ekonomi - verksamhetsstyrning</t>
+          <t>Statistisk- och maskininlärning</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -2522,19 +2522,19 @@
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE2MF</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FMI2224</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>GIK2PD</t>
+          <t>GSQ2DH</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>SQQ</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2544,18 +2544,18 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>2021-04-15</t>
+          <t>2020-02-06</t>
         </is>
       </c>
       <c r="E49" t="inlineStr"/>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Informatik</t>
+          <t>Samhällsbyggnadsteknik</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Hård infrastruktur</t>
+          <t>Introduktion till GIS</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -2565,19 +2565,19 @@
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2PD</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2DH</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>GMT2QF</t>
+          <t>FMI2229</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>MIKRODAT</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2587,18 +2587,18 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>2021-05-20</t>
+          <t>2020-06-17</t>
         </is>
       </c>
       <c r="E50" t="inlineStr"/>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Maskinteknik</t>
+          <t>Mikrodataanalys</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Finita element metoden i praktiken</t>
+          <t>Introduktion till strukturella ekvationsmodeller</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -2608,19 +2608,19 @@
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT2QF</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FMI2229</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>GIK2V4</t>
+          <t>GSQ2H7</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>SQQ</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2630,18 +2630,18 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>2022-03-01</t>
+          <t>2020-06-29</t>
         </is>
       </c>
       <c r="E51" t="inlineStr"/>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Informatik</t>
+          <t>Samhällsbyggnadsteknik</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Datasäkerhet och integritet</t>
+          <t>Gestaltad livsmiljö</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -2651,19 +2651,19 @@
       </c>
       <c r="I51" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2V4</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2H7</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>GEG2UL</t>
+          <t>GMD2GF</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2673,18 +2673,22 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>2022-03-01</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr"/>
+          <t>2020-04-08</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>2020-12-15</t>
+        </is>
+      </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Energiteknik</t>
+          <t>Matematikdidaktik</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Förnybar kraftgenerering</t>
+          <t>Matematik för lärare i åk 1-3, 30 hp (1-30). Ingår i Lärarlyftet.</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -2694,19 +2698,19 @@
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG2UL</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2GF</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>GMT2WL</t>
+          <t>GSQ2L9</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>SQQ</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2716,18 +2720,18 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>2022-06-08</t>
+          <t>2020-12-17</t>
         </is>
       </c>
       <c r="E53" t="inlineStr"/>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Maskinteknik</t>
+          <t>Samhällsbyggnadsteknik</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>3D-printing översiktskurs</t>
+          <t>Geografiska Informationssystem för samhällsplanering</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -2737,19 +2741,19 @@
       </c>
       <c r="I53" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT2WL</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2L9</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>GMD2XQ</t>
+          <t>GIE2MF</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>IEA</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2759,18 +2763,18 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>2022-09-08</t>
+          <t>2021-02-18</t>
         </is>
       </c>
       <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Matematikdidaktik</t>
+          <t>Industriell ekonomi</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Matematik för lärare i gymnasieskolan, 90 hp (1-90 hp). Ingår i lärarlyftet</t>
+          <t>Industriell ekonomi - verksamhetsstyrning</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -2780,14 +2784,14 @@
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2XQ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE2MF</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>GIK2YK</t>
+          <t>GIK2PD</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2802,7 +2806,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>2022-11-29</t>
+          <t>2021-04-15</t>
         </is>
       </c>
       <c r="E55" t="inlineStr"/>
@@ -2813,7 +2817,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Relationsdatabaser</t>
+          <t>Hård infrastruktur</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -2823,19 +2827,19 @@
       </c>
       <c r="I55" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2YK</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2PD</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>GIK2YL</t>
+          <t>GMT2QF</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2845,18 +2849,18 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>2022-11-29</t>
+          <t>2021-05-20</t>
         </is>
       </c>
       <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Informatik</t>
+          <t>Maskinteknik</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Projekt och agila arbetsmetoder</t>
+          <t>Finita element metoden i praktiken</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -2866,14 +2870,14 @@
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2YL</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT2QF</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>GIK2YN</t>
+          <t>GIK2V4</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2888,7 +2892,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>2022-11-29</t>
+          <t>2022-03-01</t>
         </is>
       </c>
       <c r="E57" t="inlineStr"/>
@@ -2899,7 +2903,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Programutvecklingsteknik</t>
+          <t>Datasäkerhet och integritet</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -2909,19 +2913,19 @@
       </c>
       <c r="I57" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2YN</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2V4</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>GIK2YP</t>
+          <t>GEG2UL</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2931,18 +2935,18 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>2022-11-29</t>
+          <t>2022-03-01</t>
         </is>
       </c>
       <c r="E58" t="inlineStr"/>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Informatik</t>
+          <t>Energiteknik</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Webbdesign</t>
+          <t>Förnybar kraftgenerering</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -2952,19 +2956,19 @@
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2YP</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG2UL</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>GIK2YR</t>
+          <t>GMT2WL</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2974,18 +2978,18 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>2022-11-29</t>
+          <t>2022-06-08</t>
         </is>
       </c>
       <c r="E59" t="inlineStr"/>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Informatik</t>
+          <t>Maskinteknik</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Designprinciper och användargränssnitt</t>
+          <t>3D-printing översiktskurs</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -2995,19 +2999,19 @@
       </c>
       <c r="I59" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2YR</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT2WL</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>GEG2ZQ</t>
+          <t>GMD2XQ</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -3017,18 +3021,18 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>2022-12-20</t>
+          <t>2022-09-08</t>
         </is>
       </c>
       <c r="E60" t="inlineStr"/>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Energiteknik</t>
+          <t>Matematikdidaktik</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Solenergi</t>
+          <t>Matematik för lärare i gymnasieskolan, 90 hp (1-90 hp). Ingår i lärarlyftet</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -3038,19 +3042,19 @@
       </c>
       <c r="I60" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG2ZQ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2XQ</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>GIK32K</t>
+          <t>FEB222K</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>ENERGIBM</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -3060,18 +3064,18 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>2023-02-07</t>
+          <t>2022-09-13</t>
         </is>
       </c>
       <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Informatik</t>
+          <t>Energisystem i byggd miljö</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Layout och typografi</t>
+          <t>Individuell litteraturkurs</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -3081,19 +3085,19 @@
       </c>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK32K</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FEB222K</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>GEG33A</t>
+          <t>FEB222L</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>ENERGIBM</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -3103,18 +3107,18 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>2023-02-23</t>
+          <t>2022-09-13</t>
         </is>
       </c>
       <c r="E62" t="inlineStr"/>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Energiteknik</t>
+          <t>Energisystem i byggd miljö</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Installation av solcellssystem</t>
+          <t>Energi och resursanvändning i den byggda miljön, del 1</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
@@ -3124,19 +3128,19 @@
       </c>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG33A</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FEB222L</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>GMD33X</t>
+          <t>FEB222M</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>ENERGIBM</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -3146,18 +3150,18 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>2023-03-17</t>
+          <t>2022-09-13</t>
         </is>
       </c>
       <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Matematikdidaktik</t>
+          <t>Energisystem i byggd miljö</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Matematik för lärare i åk 7-9</t>
+          <t>Kurs för doktorandseminarier</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -3167,19 +3171,19 @@
       </c>
       <c r="I63" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD33X</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FEB222M</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>GMD33Y</t>
+          <t>GIK2YK</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -3189,18 +3193,18 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>2023-03-17</t>
+          <t>2022-11-29</t>
         </is>
       </c>
       <c r="E64" t="inlineStr"/>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Matematikdidaktik</t>
+          <t>Informatik</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Matematik för lärare i gymnasieskolan</t>
+          <t>Relationsdatabaser</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -3210,19 +3214,19 @@
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD33Y</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2YK</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>GBY34B</t>
+          <t>GIK2YL</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>BYA</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -3232,18 +3236,18 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>2023-04-04</t>
+          <t>2022-11-29</t>
         </is>
       </c>
       <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Byggteknik</t>
+          <t>Informatik</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>Vägplanering</t>
+          <t>Projekt och agila arbetsmetoder</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
@@ -3253,14 +3257,14 @@
       </c>
       <c r="I65" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY34B</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2YL</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>GIK346</t>
+          <t>GIK2YN</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -3275,7 +3279,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>2023-04-04</t>
+          <t>2022-11-29</t>
         </is>
       </c>
       <c r="E66" t="inlineStr"/>
@@ -3286,7 +3290,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>Data Science programmering och dataanalys</t>
+          <t>Programutvecklingsteknik</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -3296,19 +3300,19 @@
       </c>
       <c r="I66" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK346</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2YN</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>GMD2H3</t>
+          <t>GIK2YP</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -3318,22 +3322,18 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>2020-06-08</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>2023-04-21</t>
-        </is>
-      </c>
+          <t>2022-11-29</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr"/>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Matematikdidaktik</t>
+          <t>Informatik</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Statistik och sannolikhetslära</t>
+          <t>Webbdesign</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -3343,19 +3343,19 @@
       </c>
       <c r="I67" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2H3</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2YP</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>GMD2H5</t>
+          <t>GIK2YR</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -3365,22 +3365,18 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>2020-06-08</t>
-        </is>
-      </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>2023-04-21</t>
-        </is>
-      </c>
+          <t>2022-11-29</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr"/>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Matematikdidaktik</t>
+          <t>Informatik</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Envariabelanalys</t>
+          <t>Designprinciper och användargränssnitt</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -3390,19 +3386,19 @@
       </c>
       <c r="I68" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2H5</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2YR</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>GIK375</t>
+          <t>GEG2ZQ</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -3412,18 +3408,18 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>2023-10-31</t>
+          <t>2022-12-20</t>
         </is>
       </c>
       <c r="E69" t="inlineStr"/>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Informatik</t>
+          <t>Energiteknik</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>Komponentdriven webbdesign</t>
+          <t>Solenergi</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
@@ -3433,14 +3429,14 @@
       </c>
       <c r="I69" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK375</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG2ZQ</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>GIK376</t>
+          <t>GIK32K</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -3455,7 +3451,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>2023-10-31</t>
+          <t>2023-02-07</t>
         </is>
       </c>
       <c r="E70" t="inlineStr"/>
@@ -3466,7 +3462,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Applikationsutveckling för webben</t>
+          <t>Layout och typografi</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
@@ -3476,19 +3472,19 @@
       </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK376</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK32K</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>GIK38G</t>
+          <t>GEG33A</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -3498,18 +3494,18 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>2023-12-19</t>
+          <t>2023-02-23</t>
         </is>
       </c>
       <c r="E71" t="inlineStr"/>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Informatik</t>
+          <t>Energiteknik</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Design av digitala tjänster</t>
+          <t>Installation av solcellssystem</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
@@ -3519,19 +3515,19 @@
       </c>
       <c r="I71" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK38G</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG33A</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>GIK38H</t>
+          <t>GMD33X</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -3541,18 +3537,18 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>2023-12-19</t>
+          <t>2023-03-17</t>
         </is>
       </c>
       <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Informatik</t>
+          <t>Matematikdidaktik</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Introduktion till IT och digitala tjänster</t>
+          <t>Matematik för lärare i åk 7-9</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
@@ -3562,19 +3558,19 @@
       </c>
       <c r="I72" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK38H</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD33X</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>GIK3BV</t>
+          <t>GMD33Y</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -3584,18 +3580,18 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>2024-05-23</t>
+          <t>2023-03-17</t>
         </is>
       </c>
       <c r="E73" t="inlineStr"/>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Informatik</t>
+          <t>Matematikdidaktik</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>E-samhället: e-förvaltning och digitala tjänster</t>
+          <t>Matematik för lärare i gymnasieskolan</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
@@ -3605,19 +3601,19 @@
       </c>
       <c r="I73" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK3BV</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD33Y</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>AEG2AY</t>
+          <t>GBY34B</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>BYA</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -3627,18 +3623,18 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>2024-06-13</t>
+          <t>2023-04-04</t>
         </is>
       </c>
       <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Energiteknik</t>
+          <t>Byggteknik</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Elektriska lagringssystem och tjänster</t>
+          <t>Vägplanering</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
@@ -3648,19 +3644,19 @@
       </c>
       <c r="I74" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2AY</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY34B</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>AEG2B5</t>
+          <t>GIK346</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -3670,18 +3666,18 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>2024-06-13</t>
+          <t>2023-04-04</t>
         </is>
       </c>
       <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Energiteknik</t>
+          <t>Informatik</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Projektkurs 3 - grupprojekt och kommunikation</t>
+          <t>Data Science programmering och dataanalys</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
@@ -3691,19 +3687,19 @@
       </c>
       <c r="I75" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2B5</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK346</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>AEG2AV</t>
+          <t>GMD2H3</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -3713,18 +3709,22 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>2024-12-12</t>
-        </is>
-      </c>
-      <c r="E76" t="inlineStr"/>
+          <t>2020-06-08</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>2023-04-21</t>
+        </is>
+      </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Energiteknik</t>
+          <t>Matematikdidaktik</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>Hållbarhet hos solenergisystem</t>
+          <t>Statistik och sannolikhetslära</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
@@ -3734,19 +3734,19 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2AV</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2H3</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>AEG2AW</t>
+          <t>GMD2H5</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -3756,18 +3756,22 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>2024-12-12</t>
-        </is>
-      </c>
-      <c r="E77" t="inlineStr"/>
+          <t>2020-06-08</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>2023-04-21</t>
+        </is>
+      </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Energiteknik</t>
+          <t>Matematikdidaktik</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>Urbana energisystem</t>
+          <t>Envariabelanalys</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
@@ -3777,19 +3781,19 @@
       </c>
       <c r="I77" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2AW</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2H5</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>AEG2AX</t>
+          <t>FEB222P</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>ENERGIBM</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -3799,18 +3803,18 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>2024-12-12</t>
+          <t>2023-10-03</t>
         </is>
       </c>
       <c r="E78" t="inlineStr"/>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Energiteknik</t>
+          <t>Energisystem i byggd miljö</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>Elnätsintegrering av förnybar kraft</t>
+          <t>Vetenskapskommunikation</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
@@ -3820,19 +3824,19 @@
       </c>
       <c r="I78" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2AX</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FEB222P</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>GMD3FX</t>
+          <t>FEB222Q</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>ENERGIBM</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -3842,18 +3846,18 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>2025-05-22</t>
+          <t>2023-10-31</t>
         </is>
       </c>
       <c r="E79" t="inlineStr"/>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Matematikdidaktik</t>
+          <t>Energisystem i byggd miljö</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>Matematikutveckling i förskoleklass och årskurs 1–3 utifrån första- och andraspråksperspektiv</t>
+          <t>Samarbetsprojekt inom energisystem</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
@@ -3863,19 +3867,19 @@
       </c>
       <c r="I79" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD3FX</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FEB222Q</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>GEG3FY</t>
+          <t>GIK375</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -3885,18 +3889,18 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>2025-05-22</t>
+          <t>2023-10-31</t>
         </is>
       </c>
       <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Energiteknik</t>
+          <t>Informatik</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>Praktik inom energiteknik</t>
+          <t>Komponentdriven webbdesign</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
@@ -3906,19 +3910,19 @@
       </c>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG3FY</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK375</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>GMT3JQ</t>
+          <t>GIK376</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -3928,18 +3932,18 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2023-10-31</t>
         </is>
       </c>
       <c r="E81" t="inlineStr"/>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Maskinteknik</t>
+          <t>Informatik</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>Mekatronik</t>
+          <t>Applikationsutveckling för webben</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
@@ -3949,19 +3953,19 @@
       </c>
       <c r="I81" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3JQ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK376</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>GMT3JR</t>
+          <t>GIK38G</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -3971,18 +3975,18 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2023-12-19</t>
         </is>
       </c>
       <c r="E82" t="inlineStr"/>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Maskinteknik</t>
+          <t>Informatik</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>Termodynamik</t>
+          <t>Design av digitala tjänster</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
@@ -3992,19 +3996,19 @@
       </c>
       <c r="I82" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3JR</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK38G</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>GMT3JY</t>
+          <t>GIK38H</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -4014,18 +4018,18 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2023-12-19</t>
         </is>
       </c>
       <c r="E83" t="inlineStr"/>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Maskinteknik</t>
+          <t>Informatik</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>Tillverkning</t>
+          <t>Introduktion till IT och digitala tjänster</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
@@ -4035,19 +4039,19 @@
       </c>
       <c r="I83" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3JY</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK38H</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>GIE3JW</t>
+          <t>GIK3BV</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>IEA</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -4057,18 +4061,18 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2024-05-23</t>
         </is>
       </c>
       <c r="E84" t="inlineStr"/>
       <c r="F84" t="inlineStr">
         <is>
-          <t>Industriell ekonomi</t>
+          <t>Informatik</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>Innovation och entreprenörskap inom assisterande teknik</t>
+          <t>E-samhället: e-förvaltning och digitala tjänster</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
@@ -4078,19 +4082,19 @@
       </c>
       <c r="I84" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE3JW</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK3BV</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>GMT3JT</t>
+          <t>AEG2AY</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -4100,18 +4104,18 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2024-06-13</t>
         </is>
       </c>
       <c r="E85" t="inlineStr"/>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Maskinteknik</t>
+          <t>Energiteknik</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>Tillämpning av regelverk för assisterande produkter</t>
+          <t>Elektriska lagringssystem och tjänster</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
@@ -4121,19 +4125,19 @@
       </c>
       <c r="I85" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3JT</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2AY</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>GMT3JU</t>
+          <t>AEG2B5</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -4143,18 +4147,18 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2024-06-13</t>
         </is>
       </c>
       <c r="E86" t="inlineStr"/>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Maskinteknik</t>
+          <t>Energiteknik</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>Smarta hem och e-hälsoteknik</t>
+          <t>Projektkurs 3 - grupprojekt och kommunikation</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
@@ -4164,19 +4168,19 @@
       </c>
       <c r="I86" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3JU</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2B5</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>GMT3JV</t>
+          <t>AEG2AV</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -4186,18 +4190,18 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2024-12-12</t>
         </is>
       </c>
       <c r="E87" t="inlineStr"/>
       <c r="F87" t="inlineStr">
         <is>
-          <t>Maskinteknik</t>
+          <t>Energiteknik</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>Assisterande robotik</t>
+          <t>Hållbarhet hos solenergisystem</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
@@ -4207,19 +4211,19 @@
       </c>
       <c r="I87" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3JV</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2AV</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>GMD3K4</t>
+          <t>AEG2AW</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -4229,33 +4233,592 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2024-12-12</t>
         </is>
       </c>
       <c r="E88" t="inlineStr"/>
       <c r="F88" t="inlineStr">
         <is>
+          <t>Energiteknik</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>Urbana energisystem</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I88" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2AW</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>AEG2AX</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>MÖY</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>IIT</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>2024-12-12</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr"/>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>Energiteknik</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>Elnätsintegrering av förnybar kraft</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I89" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2AX</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>GMD3FX</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>MDI</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>IIT</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>2025-05-22</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr"/>
+      <c r="F90" t="inlineStr">
+        <is>
           <t>Matematikdidaktik</t>
         </is>
       </c>
-      <c r="G88" t="inlineStr">
-        <is>
-          <t>Lärande och undervisning på kognitionsvetenskaplig grund</t>
-        </is>
-      </c>
-      <c r="H88" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång</t>
-        </is>
-      </c>
-      <c r="I88" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD3K4</t>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>Matematikutveckling i förskoleklass och årskurs 1–3 utifrån första- och andraspråksperspektiv</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I90" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD3FX</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>GEG3FY</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>MÖY</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>IIT</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>2025-05-22</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr"/>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>Energiteknik</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>Praktik inom energiteknik</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I91" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG3FY</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>FDA222R</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>ANALYTIC</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>IIT</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>2025-09-17</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr"/>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>Data Analytics</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>Komplexitet och operationsanalytiska metoder</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I92" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FDA222R</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>FDA222T</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>ANALYTIC</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>IIT</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>2025-09-17</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr"/>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>Data Analytics</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>Datadrivet beslutsfattande</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I93" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FDA222T</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>FDA222U</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>ANALYTIC</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>IIT</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>2025-09-17</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr"/>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>Data Analytics</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>Datainsamling och datakvalitet</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I94" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FDA222U</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>GMT3JQ</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>MTA</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>IIT</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr"/>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>Maskinteknik</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>Mekatronik</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I95" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3JQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>GMT3JR</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>MTA</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>IIT</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr"/>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Maskinteknik</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>Termodynamik</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I96" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3JR</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>GMT3JY</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>MTA</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>IIT</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr"/>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>Maskinteknik</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>Tillverkning</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I97" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3JY</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>GIE3JW</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>IEA</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>IIT</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr"/>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>Industriell ekonomi</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>Innovation och entreprenörskap inom assisterande teknik</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I98" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE3JW</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>GMT3JT</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>MTA</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>IIT</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr"/>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>Maskinteknik</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>Tillämpning av regelverk för assisterande produkter</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I99" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3JT</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>GMT3JU</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>MTA</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>IIT</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr"/>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>Maskinteknik</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>Smarta hem och e-hälsoteknik</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I100" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3JU</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>GMT3JV</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>MTA</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>IIT</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr"/>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>Maskinteknik</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>Assisterande robotik</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I101" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3JV</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I88"/>
+  <autoFilter ref="A1:I101"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I2" r:id="rId2"/>
@@ -4431,6 +4994,32 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I87" r:id="rId172"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A88" r:id="rId173"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I88" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A89" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I89" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A90" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I90" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A91" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I91" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A92" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I92" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A93" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I93" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A94" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I94" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A95" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I95" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A96" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I96" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A97" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I97" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A98" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I98" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A99" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I99" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A100" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I100" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A101" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I101" r:id="rId200"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update educational program documents and add new course plans for GPG3KA and GPG3KB
- Removed empty headings in HEELA.md, HMILA.md, HSVAA.md, HTESA.md, LG79A.md, LGGYA.md, LL46A.md, LLF3A.md, LLL3A.md, LLL6A.md, LLP6A.md, LU79A.md, LUGYA.md, and LYSLA.md.
- Added new course plan for "Didaktik och ledarskap för ämneslärare inriktning årskurs 7-9 (inkl 7,5 hp VFU)" (GPG3KA).
- Added new course plan for "Didaktik och ledarskap för ämneslärare inriktning gymnasieskolan (inkl 7,5 hp VFU)" (GPG3KB).
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/01 IIT/Analys/Vilande kursplaner.xlsx
+++ b/vault-dalarna-university/01 IIT/Analys/Vilande kursplaner.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Vilande kursplaner" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Vilande kursplaner'!$A$1:$I$104</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Vilande kursplaner'!$A$1:$I$112</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I104"/>
+  <dimension ref="A1:I112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1751,12 +1751,12 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>MT1074</t>
+          <t>EG3022</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1766,18 +1766,18 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>2018-02-15</t>
+          <t>2018-01-25</t>
         </is>
       </c>
       <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Maskinteknik</t>
+          <t>Energiteknik</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Maskinelement</t>
+          <t>Examensarbete för magisterexamen i solenergiteknik</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -1787,19 +1787,19 @@
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1074</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3022</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>GMT228</t>
+          <t>ET1029</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>ETA</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1809,18 +1809,18 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>2018-04-05</t>
+          <t>2018-02-13</t>
         </is>
       </c>
       <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Maskinteknik</t>
+          <t>Elektroteknik</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Produktutvecklingsmetoder</t>
+          <t>Styr- och reglerteknik</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -1830,19 +1830,19 @@
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT228</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ET1029</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>AEG225</t>
+          <t>MT1074</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1852,18 +1852,18 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>2018-05-24</t>
+          <t>2018-02-15</t>
         </is>
       </c>
       <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Energiteknik</t>
+          <t>Maskinteknik</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Solenergins ekonomi</t>
+          <t>Maskinelement</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -1873,19 +1873,19 @@
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG225</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1074</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>GSQ23J</t>
+          <t>GMT228</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>SQQ</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1895,18 +1895,18 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>2018-05-24</t>
+          <t>2018-04-05</t>
         </is>
       </c>
       <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Samhällsbyggnadsteknik</t>
+          <t>Maskinteknik</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Befolkning och sociala perspektiv</t>
+          <t>Produktutvecklingsmetoder</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -1916,19 +1916,19 @@
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ23J</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT228</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>GSQ23K</t>
+          <t>AEG225</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>SQQ</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1938,18 +1938,18 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>2018-06-14</t>
+          <t>2018-05-24</t>
         </is>
       </c>
       <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Samhällsbyggnadsteknik</t>
+          <t>Energiteknik</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Planeringsprojekt</t>
+          <t>Solenergins ekonomi</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -1959,14 +1959,14 @@
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ23K</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG225</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>GSQ25J</t>
+          <t>GSQ23J</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1981,7 +1981,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>2018-10-29</t>
+          <t>2018-05-24</t>
         </is>
       </c>
       <c r="E36" t="inlineStr"/>
@@ -1992,7 +1992,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Vetenskaplig metod</t>
+          <t>Befolkning och sociala perspektiv</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -2002,14 +2002,14 @@
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25J</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ23J</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>GSQ25K</t>
+          <t>GSQ23K</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2024,7 +2024,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>2018-11-08</t>
+          <t>2018-06-14</t>
         </is>
       </c>
       <c r="E37" t="inlineStr"/>
@@ -2035,7 +2035,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Stadsbyggnad</t>
+          <t>Planeringsprojekt</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -2045,19 +2045,19 @@
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25K</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ23K</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>GMT25Z</t>
+          <t>GSQ25J</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>SQQ</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2067,18 +2067,18 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>2019-01-31</t>
+          <t>2018-10-29</t>
         </is>
       </c>
       <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Maskinteknik</t>
+          <t>Samhällsbyggnadsteknik</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Examensarbete Högskoleingenjör Maskinteknik</t>
+          <t>Vetenskaplig metod</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -2088,19 +2088,19 @@
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT25Z</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25J</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>AEG22R</t>
+          <t>GSQ25K</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>SQQ</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2110,18 +2110,18 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>2019-01-31</t>
+          <t>2018-11-08</t>
         </is>
       </c>
       <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Energiteknik</t>
+          <t>Samhällsbyggnadsteknik</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Tillämpad solenergiteknik</t>
+          <t>Stadsbyggnad</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -2131,19 +2131,19 @@
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG22R</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25K</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>GIE26P</t>
+          <t>GMT25Z</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>IEA</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2153,18 +2153,18 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>2019-02-21</t>
+          <t>2019-01-31</t>
         </is>
       </c>
       <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Industriell ekonomi</t>
+          <t>Maskinteknik</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Industriell ekonomi - grundläggande kurs</t>
+          <t>Examensarbete Högskoleingenjör Maskinteknik</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -2174,19 +2174,19 @@
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE26P</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT25Z</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>GIK289</t>
+          <t>AEG22R</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2196,18 +2196,18 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>2019-02-21</t>
+          <t>2019-01-31</t>
         </is>
       </c>
       <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Informatik</t>
+          <t>Energiteknik</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Objektorienterad programmering och problemlösning</t>
+          <t>Tillämpad solenergiteknik</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -2217,19 +2217,19 @@
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK289</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG22R</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>GEG26J</t>
+          <t>GIE26P</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>IEA</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2245,12 +2245,12 @@
       <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Energiteknik</t>
+          <t>Industriell ekonomi</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Vetenskaplig kommunikation</t>
+          <t>Industriell ekonomi - grundläggande kurs</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -2260,19 +2260,19 @@
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG26J</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE26P</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>AEG233</t>
+          <t>GIK289</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2282,18 +2282,18 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>2019-06-05</t>
+          <t>2019-02-21</t>
         </is>
       </c>
       <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Energiteknik</t>
+          <t>Informatik</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Solel</t>
+          <t>Objektorienterad programmering och problemlösning</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -2303,19 +2303,19 @@
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG233</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK289</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>GIE29N</t>
+          <t>GEG26J</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>IEA</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2325,18 +2325,18 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>2019-06-13</t>
+          <t>2019-02-21</t>
         </is>
       </c>
       <c r="E44" t="inlineStr"/>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Industriell ekonomi</t>
+          <t>Energiteknik</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Industriell ekonomi - Processer och projektledning</t>
+          <t>Vetenskaplig kommunikation</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -2346,19 +2346,19 @@
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE29N</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG26J</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>GMD2BH</t>
+          <t>AEG233</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2368,22 +2368,18 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>2019-08-29</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>2019-09-19</t>
-        </is>
-      </c>
+          <t>2019-06-05</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr"/>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Matematikdidaktik</t>
+          <t>Energiteknik</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Matematikdidaktik I</t>
+          <t>Solel</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -2393,19 +2389,19 @@
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2BH</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG233</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>FMI2222</t>
+          <t>GIE29N</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>MIKRODAT</t>
+          <t>IEA</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2415,18 +2411,18 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>2019-10-03</t>
+          <t>2019-06-13</t>
         </is>
       </c>
       <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Mikrodataanalys</t>
+          <t>Industriell ekonomi</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Ledarskapets ekonomi för forskarstuderande</t>
+          <t>Industriell ekonomi - Processer och projektledning</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -2436,19 +2432,19 @@
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FMI2222</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE29N</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>BEG222</t>
+          <t>GMD2BH</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2458,18 +2454,22 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>2019-10-17</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr"/>
+          <t>2019-08-29</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>2019-09-19</t>
+        </is>
+      </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Energiteknik</t>
+          <t>Matematikdidaktik</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Grundläggande forskningsmetodik</t>
+          <t>Matematikdidaktik I</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -2479,14 +2479,14 @@
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BEG222</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2BH</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>FMI2224</t>
+          <t>FMI2222</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2501,7 +2501,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>2019-10-29</t>
+          <t>2019-10-03</t>
         </is>
       </c>
       <c r="E48" t="inlineStr"/>
@@ -2512,7 +2512,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Statistisk- och maskininlärning</t>
+          <t>Ledarskapets ekonomi för forskarstuderande</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -2522,19 +2522,19 @@
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FMI2224</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FMI2222</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>GSQ2DH</t>
+          <t>BEG222</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>SQQ</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2544,18 +2544,18 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>2020-02-06</t>
+          <t>2019-10-17</t>
         </is>
       </c>
       <c r="E49" t="inlineStr"/>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Samhällsbyggnadsteknik</t>
+          <t>Energiteknik</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Introduktion till GIS</t>
+          <t>Grundläggande forskningsmetodik</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -2565,14 +2565,14 @@
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2DH</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BEG222</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>FMI2229</t>
+          <t>FMI2224</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2587,7 +2587,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>2020-06-17</t>
+          <t>2019-10-29</t>
         </is>
       </c>
       <c r="E50" t="inlineStr"/>
@@ -2598,7 +2598,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Introduktion till strukturella ekvationsmodeller</t>
+          <t>Statistisk- och maskininlärning</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -2608,14 +2608,14 @@
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FMI2229</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FMI2224</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>GSQ2H7</t>
+          <t>GSQ2DH</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2630,7 +2630,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>2020-06-29</t>
+          <t>2020-02-06</t>
         </is>
       </c>
       <c r="E51" t="inlineStr"/>
@@ -2641,7 +2641,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Gestaltad livsmiljö</t>
+          <t>Introduktion till GIS</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -2651,19 +2651,19 @@
       </c>
       <c r="I51" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2H7</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2DH</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>GMD2GF</t>
+          <t>FMI2229</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>MIKRODAT</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2673,22 +2673,18 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>2020-04-08</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>2020-12-15</t>
-        </is>
-      </c>
+          <t>2020-06-17</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Matematikdidaktik</t>
+          <t>Mikrodataanalys</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Matematik för lärare i åk 1-3, 30 hp (1-30). Ingår i Lärarlyftet.</t>
+          <t>Introduktion till strukturella ekvationsmodeller</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -2698,14 +2694,14 @@
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2GF</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FMI2229</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>GSQ2L9</t>
+          <t>GSQ2H7</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2720,7 +2716,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>2020-12-17</t>
+          <t>2020-06-29</t>
         </is>
       </c>
       <c r="E53" t="inlineStr"/>
@@ -2731,7 +2727,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Geografiska Informationssystem för samhällsplanering</t>
+          <t>Gestaltad livsmiljö</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -2741,19 +2737,19 @@
       </c>
       <c r="I53" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2L9</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2H7</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>GIE2MF</t>
+          <t>GMD2GF</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>IEA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2763,18 +2759,22 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>2021-02-18</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr"/>
+          <t>2020-04-08</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>2020-12-15</t>
+        </is>
+      </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Industriell ekonomi</t>
+          <t>Matematikdidaktik</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Industriell ekonomi - verksamhetsstyrning</t>
+          <t>Matematik för lärare i åk 1-3, 30 hp (1-30). Ingår i Lärarlyftet.</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -2784,19 +2784,19 @@
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE2MF</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2GF</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>GIK2PD</t>
+          <t>GSQ2L9</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>SQQ</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2806,18 +2806,18 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>2021-04-15</t>
+          <t>2020-12-17</t>
         </is>
       </c>
       <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Informatik</t>
+          <t>Samhällsbyggnadsteknik</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Hård infrastruktur</t>
+          <t>Geografiska Informationssystem för samhällsplanering</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -2827,19 +2827,19 @@
       </c>
       <c r="I55" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2PD</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2L9</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>GMT2QF</t>
+          <t>GIE2MF</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>IEA</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2849,18 +2849,18 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>2021-05-20</t>
+          <t>2021-02-18</t>
         </is>
       </c>
       <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Maskinteknik</t>
+          <t>Industriell ekonomi</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Finita element metoden i praktiken</t>
+          <t>Industriell ekonomi - verksamhetsstyrning</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -2870,14 +2870,14 @@
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT2QF</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE2MF</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>GIK2V4</t>
+          <t>GIK2PD</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2892,7 +2892,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>2022-03-01</t>
+          <t>2021-04-15</t>
         </is>
       </c>
       <c r="E57" t="inlineStr"/>
@@ -2903,7 +2903,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Datasäkerhet och integritet</t>
+          <t>Hård infrastruktur</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -2913,19 +2913,19 @@
       </c>
       <c r="I57" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2V4</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2PD</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>GEG2UL</t>
+          <t>GMT2QF</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2935,18 +2935,18 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>2022-03-01</t>
+          <t>2021-05-20</t>
         </is>
       </c>
       <c r="E58" t="inlineStr"/>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Energiteknik</t>
+          <t>Maskinteknik</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Förnybar kraftgenerering</t>
+          <t>Finita element metoden i praktiken</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -2956,19 +2956,19 @@
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG2UL</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT2QF</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>GMT2WL</t>
+          <t>GIK2QZ</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2978,18 +2978,18 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>2022-06-08</t>
+          <t>2021-08-24</t>
         </is>
       </c>
       <c r="E59" t="inlineStr"/>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Maskinteknik</t>
+          <t>Informatik</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>3D-printing översiktskurs</t>
+          <t>Visuell identitet</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -2999,19 +2999,19 @@
       </c>
       <c r="I59" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT2WL</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2QZ</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>GMD2XQ</t>
+          <t>GIK2V4</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -3021,18 +3021,18 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>2022-09-08</t>
+          <t>2022-03-01</t>
         </is>
       </c>
       <c r="E60" t="inlineStr"/>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Matematikdidaktik</t>
+          <t>Informatik</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Matematik för lärare i gymnasieskolan, 90 hp (1-90 hp). Ingår i lärarlyftet</t>
+          <t>Datasäkerhet och integritet</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -3042,19 +3042,19 @@
       </c>
       <c r="I60" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2XQ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2V4</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>FEB222K</t>
+          <t>GEG2UL</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>ENERGIBM</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -3064,18 +3064,18 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>2022-09-13</t>
+          <t>2022-03-01</t>
         </is>
       </c>
       <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Energisystem i byggd miljö</t>
+          <t>Energiteknik</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Individuell litteraturkurs</t>
+          <t>Förnybar kraftgenerering</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -3085,19 +3085,19 @@
       </c>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FEB222K</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG2UL</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>FEB222L</t>
+          <t>GMT2WL</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>ENERGIBM</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -3107,18 +3107,18 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>2022-09-13</t>
+          <t>2022-06-08</t>
         </is>
       </c>
       <c r="E62" t="inlineStr"/>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Energisystem i byggd miljö</t>
+          <t>Maskinteknik</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Energi och resursanvändning i den byggda miljön, del 1</t>
+          <t>3D-printing översiktskurs</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
@@ -3128,19 +3128,19 @@
       </c>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FEB222L</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT2WL</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>FEB222M</t>
+          <t>GMD2XQ</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>ENERGIBM</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -3150,18 +3150,18 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>2022-09-13</t>
+          <t>2022-09-08</t>
         </is>
       </c>
       <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Energisystem i byggd miljö</t>
+          <t>Matematikdidaktik</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Kurs för doktorandseminarier</t>
+          <t>Matematik för lärare i gymnasieskolan, 90 hp (1-90 hp). Ingår i lärarlyftet</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -3171,19 +3171,19 @@
       </c>
       <c r="I63" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FEB222M</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2XQ</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>GIK2YK</t>
+          <t>FEB222K</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>ENERGIBM</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -3193,18 +3193,18 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>2022-11-29</t>
+          <t>2022-09-13</t>
         </is>
       </c>
       <c r="E64" t="inlineStr"/>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Informatik</t>
+          <t>Energisystem i byggd miljö</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Relationsdatabaser</t>
+          <t>Individuell litteraturkurs</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -3214,19 +3214,19 @@
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2YK</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FEB222K</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>GIK2YL</t>
+          <t>FEB222L</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>ENERGIBM</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -3236,18 +3236,18 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>2022-11-29</t>
+          <t>2022-09-13</t>
         </is>
       </c>
       <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Informatik</t>
+          <t>Energisystem i byggd miljö</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>Projekt och agila arbetsmetoder</t>
+          <t>Energi och resursanvändning i den byggda miljön, del 1</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
@@ -3257,19 +3257,19 @@
       </c>
       <c r="I65" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2YL</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FEB222L</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>GIK2YN</t>
+          <t>FEB222M</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>ENERGIBM</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -3279,18 +3279,18 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>2022-11-29</t>
+          <t>2022-09-13</t>
         </is>
       </c>
       <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Informatik</t>
+          <t>Energisystem i byggd miljö</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>Programutvecklingsteknik</t>
+          <t>Kurs för doktorandseminarier</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -3300,14 +3300,14 @@
       </c>
       <c r="I66" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2YN</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FEB222M</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>GIK2YP</t>
+          <t>GIK2YK</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -3333,7 +3333,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Webbdesign</t>
+          <t>Relationsdatabaser</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -3343,14 +3343,14 @@
       </c>
       <c r="I67" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2YP</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2YK</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>GIK2YR</t>
+          <t>GIK2YL</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -3376,7 +3376,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Designprinciper och användargränssnitt</t>
+          <t>Projekt och agila arbetsmetoder</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -3386,19 +3386,19 @@
       </c>
       <c r="I68" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2YR</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2YL</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>GEG2ZQ</t>
+          <t>GIK2YN</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -3408,18 +3408,18 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>2022-12-20</t>
+          <t>2022-11-29</t>
         </is>
       </c>
       <c r="E69" t="inlineStr"/>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Energiteknik</t>
+          <t>Informatik</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>Solenergi</t>
+          <t>Programutvecklingsteknik</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
@@ -3429,14 +3429,14 @@
       </c>
       <c r="I69" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG2ZQ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2YN</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>GIK32K</t>
+          <t>GIK2YP</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -3451,7 +3451,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>2023-02-07</t>
+          <t>2022-11-29</t>
         </is>
       </c>
       <c r="E70" t="inlineStr"/>
@@ -3462,7 +3462,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Layout och typografi</t>
+          <t>Webbdesign</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
@@ -3472,19 +3472,19 @@
       </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK32K</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2YP</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>GEG33A</t>
+          <t>GIK2YR</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -3494,18 +3494,18 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>2023-02-23</t>
+          <t>2022-11-29</t>
         </is>
       </c>
       <c r="E71" t="inlineStr"/>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Energiteknik</t>
+          <t>Informatik</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Installation av solcellssystem</t>
+          <t>Designprinciper och användargränssnitt</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
@@ -3515,19 +3515,19 @@
       </c>
       <c r="I71" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG33A</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2YR</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>GMD33X</t>
+          <t>GEG2ZQ</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -3537,18 +3537,18 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>2023-03-17</t>
+          <t>2022-12-20</t>
         </is>
       </c>
       <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Matematikdidaktik</t>
+          <t>Energiteknik</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Matematik för lärare i åk 7-9</t>
+          <t>Solenergi</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
@@ -3558,19 +3558,19 @@
       </c>
       <c r="I72" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD33X</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG2ZQ</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>GMD33Y</t>
+          <t>GIK32K</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -3580,18 +3580,18 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>2023-03-17</t>
+          <t>2023-02-07</t>
         </is>
       </c>
       <c r="E73" t="inlineStr"/>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Matematikdidaktik</t>
+          <t>Informatik</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>Matematik för lärare i gymnasieskolan</t>
+          <t>Layout och typografi</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
@@ -3601,19 +3601,19 @@
       </c>
       <c r="I73" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD33Y</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK32K</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>GBY34B</t>
+          <t>GEG33A</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>BYA</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -3623,18 +3623,18 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>2023-04-04</t>
+          <t>2023-02-23</t>
         </is>
       </c>
       <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Byggteknik</t>
+          <t>Energiteknik</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Vägplanering</t>
+          <t>Installation av solcellssystem</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
@@ -3644,19 +3644,19 @@
       </c>
       <c r="I74" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY34B</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG33A</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>GIK346</t>
+          <t>GMD33X</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -3666,18 +3666,18 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>2023-04-04</t>
+          <t>2023-03-17</t>
         </is>
       </c>
       <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Informatik</t>
+          <t>Matematikdidaktik</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Data Science programmering och dataanalys</t>
+          <t>Matematik för lärare i åk 7-9</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
@@ -3687,14 +3687,14 @@
       </c>
       <c r="I75" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK346</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD33X</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>GMD2H3</t>
+          <t>GMD33Y</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -3709,14 +3709,10 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>2020-06-08</t>
-        </is>
-      </c>
-      <c r="E76" t="inlineStr">
-        <is>
-          <t>2023-04-21</t>
-        </is>
-      </c>
+          <t>2023-03-17</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr"/>
       <c r="F76" t="inlineStr">
         <is>
           <t>Matematikdidaktik</t>
@@ -3724,7 +3720,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>Statistik och sannolikhetslära</t>
+          <t>Matematik för lärare i gymnasieskolan</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
@@ -3734,19 +3730,19 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2H3</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD33Y</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>GMD2H5</t>
+          <t>GBY34B</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>BYA</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -3756,22 +3752,18 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>2020-06-08</t>
-        </is>
-      </c>
-      <c r="E77" t="inlineStr">
-        <is>
-          <t>2023-04-21</t>
-        </is>
-      </c>
+          <t>2023-04-04</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr"/>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Matematikdidaktik</t>
+          <t>Byggteknik</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>Envariabelanalys</t>
+          <t>Vägplanering</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
@@ -3781,19 +3773,19 @@
       </c>
       <c r="I77" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2H5</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY34B</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>FEB222P</t>
+          <t>GFY345</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>ENERGIBM</t>
+          <t>FYA</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -3803,18 +3795,18 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>2023-10-03</t>
+          <t>2023-04-04</t>
         </is>
       </c>
       <c r="E78" t="inlineStr"/>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Energisystem i byggd miljö</t>
+          <t>Fysik</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>Vetenskapskommunikation</t>
+          <t>Fysik för tekniker</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
@@ -3824,19 +3816,19 @@
       </c>
       <c r="I78" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FEB222P</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GFY345</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>FEB222Q</t>
+          <t>GIK346</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>ENERGIBM</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -3846,18 +3838,18 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>2023-10-31</t>
+          <t>2023-04-04</t>
         </is>
       </c>
       <c r="E79" t="inlineStr"/>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Energisystem i byggd miljö</t>
+          <t>Informatik</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>Samarbetsprojekt inom energisystem</t>
+          <t>Data Science programmering och dataanalys</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
@@ -3867,19 +3859,19 @@
       </c>
       <c r="I79" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FEB222Q</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK346</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>GIK375</t>
+          <t>GMD2H3</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -3889,18 +3881,22 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>2023-10-31</t>
-        </is>
-      </c>
-      <c r="E80" t="inlineStr"/>
+          <t>2020-06-08</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>2023-04-21</t>
+        </is>
+      </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Informatik</t>
+          <t>Matematikdidaktik</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>Komponentdriven webbdesign</t>
+          <t>Statistik och sannolikhetslära</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
@@ -3910,19 +3906,19 @@
       </c>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK375</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2H3</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>GIK376</t>
+          <t>GMD2H5</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -3932,18 +3928,22 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>2023-10-31</t>
-        </is>
-      </c>
-      <c r="E81" t="inlineStr"/>
+          <t>2020-06-08</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>2023-04-21</t>
+        </is>
+      </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Informatik</t>
+          <t>Matematikdidaktik</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>Applikationsutveckling för webben</t>
+          <t>Envariabelanalys</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
@@ -3953,19 +3953,19 @@
       </c>
       <c r="I81" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK376</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2H5</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>GIK38G</t>
+          <t>FEB222P</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>ENERGIBM</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -3975,18 +3975,18 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>2023-12-19</t>
+          <t>2023-10-03</t>
         </is>
       </c>
       <c r="E82" t="inlineStr"/>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Informatik</t>
+          <t>Energisystem i byggd miljö</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>Design av digitala tjänster</t>
+          <t>Vetenskapskommunikation</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
@@ -3996,19 +3996,19 @@
       </c>
       <c r="I82" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK38G</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FEB222P</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>GIK38H</t>
+          <t>GET36T</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>ETA</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -4018,18 +4018,18 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>2023-12-19</t>
+          <t>2023-10-03</t>
         </is>
       </c>
       <c r="E83" t="inlineStr"/>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Informatik</t>
+          <t>Elektroteknik</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>Introduktion till IT och digitala tjänster</t>
+          <t>Ellära</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
@@ -4039,14 +4039,14 @@
       </c>
       <c r="I83" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK38H</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GET36T</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>GIK3BV</t>
+          <t>GIK36R</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -4061,7 +4061,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>2024-05-23</t>
+          <t>2023-10-03</t>
         </is>
       </c>
       <c r="E84" t="inlineStr"/>
@@ -4072,7 +4072,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>E-samhället: e-förvaltning och digitala tjänster</t>
+          <t>Applikationsutveckling och testning</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
@@ -4082,19 +4082,19 @@
       </c>
       <c r="I84" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK3BV</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK36R</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>AEG2AY</t>
+          <t>FEB222Q</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>ENERGIBM</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -4104,18 +4104,18 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>2024-06-13</t>
+          <t>2023-10-31</t>
         </is>
       </c>
       <c r="E85" t="inlineStr"/>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Energiteknik</t>
+          <t>Energisystem i byggd miljö</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>Elektriska lagringssystem och tjänster</t>
+          <t>Samarbetsprojekt inom energisystem</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
@@ -4125,19 +4125,19 @@
       </c>
       <c r="I85" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2AY</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FEB222Q</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>AEG2B5</t>
+          <t>GIK375</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -4147,18 +4147,18 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>2024-06-13</t>
+          <t>2023-10-31</t>
         </is>
       </c>
       <c r="E86" t="inlineStr"/>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Energiteknik</t>
+          <t>Informatik</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>Projektkurs 3 - grupprojekt och kommunikation</t>
+          <t>Komponentdriven webbdesign</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
@@ -4168,19 +4168,19 @@
       </c>
       <c r="I86" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2B5</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK375</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>AEG2AV</t>
+          <t>GIK376</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -4190,18 +4190,18 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>2024-12-12</t>
+          <t>2023-10-31</t>
         </is>
       </c>
       <c r="E87" t="inlineStr"/>
       <c r="F87" t="inlineStr">
         <is>
-          <t>Energiteknik</t>
+          <t>Informatik</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>Hållbarhet hos solenergisystem</t>
+          <t>Applikationsutveckling för webben</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
@@ -4211,19 +4211,19 @@
       </c>
       <c r="I87" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2AV</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK376</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>AEG2AW</t>
+          <t>GIK377</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -4233,18 +4233,18 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>2024-12-12</t>
+          <t>2023-10-31</t>
         </is>
       </c>
       <c r="E88" t="inlineStr"/>
       <c r="F88" t="inlineStr">
         <is>
-          <t>Energiteknik</t>
+          <t>Informatik</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>Urbana energisystem</t>
+          <t>Utveckling av digitala tjänster</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
@@ -4254,19 +4254,19 @@
       </c>
       <c r="I88" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2AW</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK377</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>AEG2AX</t>
+          <t>GIK38G</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -4276,18 +4276,18 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>2024-12-12</t>
+          <t>2023-12-19</t>
         </is>
       </c>
       <c r="E89" t="inlineStr"/>
       <c r="F89" t="inlineStr">
         <is>
-          <t>Energiteknik</t>
+          <t>Informatik</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>Elnätsintegrering av förnybar kraft</t>
+          <t>Design av digitala tjänster</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
@@ -4297,19 +4297,19 @@
       </c>
       <c r="I89" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2AX</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK38G</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>GMD3FX</t>
+          <t>GIK38H</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -4319,18 +4319,18 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>2025-05-22</t>
+          <t>2023-12-19</t>
         </is>
       </c>
       <c r="E90" t="inlineStr"/>
       <c r="F90" t="inlineStr">
         <is>
-          <t>Matematikdidaktik</t>
+          <t>Informatik</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>Matematikutveckling i förskoleklass och årskurs 1–3 utifrån första- och andraspråksperspektiv</t>
+          <t>Introduktion till IT och digitala tjänster</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
@@ -4340,19 +4340,19 @@
       </c>
       <c r="I90" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD3FX</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK38H</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>GEG3FY</t>
+          <t>GIK3BV</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -4362,18 +4362,18 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>2025-05-22</t>
+          <t>2024-05-23</t>
         </is>
       </c>
       <c r="E91" t="inlineStr"/>
       <c r="F91" t="inlineStr">
         <is>
-          <t>Energiteknik</t>
+          <t>Informatik</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>Praktik inom energiteknik</t>
+          <t>E-samhället: e-förvaltning och digitala tjänster</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
@@ -4383,19 +4383,19 @@
       </c>
       <c r="I91" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG3FY</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK3BV</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>FDA222R</t>
+          <t>AEG2AY</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>ANALYTIC</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -4405,18 +4405,18 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>2025-09-17</t>
+          <t>2024-06-13</t>
         </is>
       </c>
       <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr">
         <is>
-          <t>Data Analytics</t>
+          <t>Energiteknik</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>Komplexitet och operationsanalytiska metoder</t>
+          <t>Elektriska lagringssystem och tjänster</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
@@ -4426,19 +4426,19 @@
       </c>
       <c r="I92" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FDA222R</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2AY</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>FDA222T</t>
+          <t>AEG2B5</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>ANALYTIC</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -4448,18 +4448,18 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>2025-09-17</t>
+          <t>2024-06-13</t>
         </is>
       </c>
       <c r="E93" t="inlineStr"/>
       <c r="F93" t="inlineStr">
         <is>
-          <t>Data Analytics</t>
+          <t>Energiteknik</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>Datadrivet beslutsfattande</t>
+          <t>Projektkurs 3 - grupprojekt och kommunikation</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
@@ -4469,19 +4469,19 @@
       </c>
       <c r="I93" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FDA222T</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2B5</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>FDA222U</t>
+          <t>AEG2AV</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>ANALYTIC</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -4491,18 +4491,18 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>2025-09-17</t>
+          <t>2024-12-12</t>
         </is>
       </c>
       <c r="E94" t="inlineStr"/>
       <c r="F94" t="inlineStr">
         <is>
-          <t>Data Analytics</t>
+          <t>Energiteknik</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>Datainsamling och datakvalitet</t>
+          <t>Hållbarhet hos solenergisystem</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
@@ -4512,19 +4512,19 @@
       </c>
       <c r="I94" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FDA222U</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2AV</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>GMT3JQ</t>
+          <t>AEG2AW</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -4534,18 +4534,18 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2024-12-12</t>
         </is>
       </c>
       <c r="E95" t="inlineStr"/>
       <c r="F95" t="inlineStr">
         <is>
-          <t>Maskinteknik</t>
+          <t>Energiteknik</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>Mekatronik</t>
+          <t>Urbana energisystem</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
@@ -4555,19 +4555,19 @@
       </c>
       <c r="I95" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3JQ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2AW</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>GMT3JR</t>
+          <t>AEG2AX</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -4577,18 +4577,18 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2024-12-12</t>
         </is>
       </c>
       <c r="E96" t="inlineStr"/>
       <c r="F96" t="inlineStr">
         <is>
-          <t>Maskinteknik</t>
+          <t>Energiteknik</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>Termodynamik</t>
+          <t>Elnätsintegrering av förnybar kraft</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
@@ -4598,19 +4598,19 @@
       </c>
       <c r="I96" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3JR</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2AX</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>GMT3JY</t>
+          <t>GMD3FX</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -4620,18 +4620,18 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2025-05-22</t>
         </is>
       </c>
       <c r="E97" t="inlineStr"/>
       <c r="F97" t="inlineStr">
         <is>
-          <t>Maskinteknik</t>
+          <t>Matematikdidaktik</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>Tillverkning</t>
+          <t>Matematikutveckling i förskoleklass och årskurs 1–3 utifrån första- och andraspråksperspektiv</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
@@ -4641,19 +4641,19 @@
       </c>
       <c r="I97" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3JY</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD3FX</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>GIE3JW</t>
+          <t>GEG3FY</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>IEA</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -4663,18 +4663,18 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2025-05-22</t>
         </is>
       </c>
       <c r="E98" t="inlineStr"/>
       <c r="F98" t="inlineStr">
         <is>
-          <t>Industriell ekonomi</t>
+          <t>Energiteknik</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>Innovation och entreprenörskap inom assisterande teknik</t>
+          <t>Praktik inom energiteknik</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
@@ -4684,19 +4684,19 @@
       </c>
       <c r="I98" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE3JW</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG3FY</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>GMT3JT</t>
+          <t>FDA222R</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>ANALYTIC</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -4706,18 +4706,18 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2025-09-17</t>
         </is>
       </c>
       <c r="E99" t="inlineStr"/>
       <c r="F99" t="inlineStr">
         <is>
-          <t>Maskinteknik</t>
+          <t>Data Analytics</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>Tillämpning av regelverk för assisterande produkter</t>
+          <t>Komplexitet och operationsanalytiska metoder</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
@@ -4727,19 +4727,19 @@
       </c>
       <c r="I99" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3JT</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FDA222R</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>GMT3JU</t>
+          <t>FDA222S</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>ANALYTIC</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -4749,18 +4749,18 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2025-09-17</t>
         </is>
       </c>
       <c r="E100" t="inlineStr"/>
       <c r="F100" t="inlineStr">
         <is>
-          <t>Maskinteknik</t>
+          <t>Data Analytics</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>Smarta hem och e-hälsoteknik</t>
+          <t>Statistisk inlärning och maskininlärning</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
@@ -4770,19 +4770,19 @@
       </c>
       <c r="I100" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3JU</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FDA222S</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>GMT3JV</t>
+          <t>FDA222T</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>ANALYTIC</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -4792,18 +4792,18 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2025-09-17</t>
         </is>
       </c>
       <c r="E101" t="inlineStr"/>
       <c r="F101" t="inlineStr">
         <is>
-          <t>Maskinteknik</t>
+          <t>Data Analytics</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>Assisterande robotik</t>
+          <t>Datadrivet beslutsfattande</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
@@ -4813,19 +4813,19 @@
       </c>
       <c r="I101" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3JV</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FDA222T</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>BMA229</t>
+          <t>FDA222U</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>MAA</t>
+          <t>ANALYTIC</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -4835,18 +4835,18 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2025-09-17</t>
         </is>
       </c>
       <c r="E102" t="inlineStr"/>
       <c r="F102" t="inlineStr">
         <is>
-          <t>Matematik</t>
+          <t>Data Analytics</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>Basmatematik 2</t>
+          <t>Datainsamling och datakvalitet</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
@@ -4856,14 +4856,14 @@
       </c>
       <c r="I102" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BMA229</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FDA222U</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>GMT3K5</t>
+          <t>GMT3JQ</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -4878,7 +4878,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="E103" t="inlineStr"/>
@@ -4889,7 +4889,7 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>Examensarbete i assisterande teknik med inriktning mot maskinteknik</t>
+          <t>Mekatronik</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
@@ -4899,14 +4899,14 @@
       </c>
       <c r="I103" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3K5</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3JQ</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>GMT3K6</t>
+          <t>GMT3JR</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -4921,7 +4921,7 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="E104" t="inlineStr"/>
@@ -4932,22 +4932,366 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
+          <t>Termodynamik</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I104" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3JR</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>GMT3JY</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>MTA</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>IIT</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr"/>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>Maskinteknik</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>Tillverkning</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I105" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3JY</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>GIE3JW</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>IEA</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>IIT</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr"/>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>Industriell ekonomi</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>Innovation och entreprenörskap inom assisterande teknik</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I106" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE3JW</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>GMT3JT</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>MTA</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>IIT</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr"/>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>Maskinteknik</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>Tillämpning av regelverk för assisterande produkter</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I107" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3JT</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>GMT3JU</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>MTA</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>IIT</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr"/>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>Maskinteknik</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>Smarta hem och e-hälsoteknik</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I108" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3JU</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>GMT3JV</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>MTA</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>IIT</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr"/>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>Maskinteknik</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>Assisterande robotik</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I109" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3JV</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>BMA229</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>MAA</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>IIT</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr"/>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>Matematik</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>Basmatematik 2</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I110" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BMA229</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>GMT3K5</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>MTA</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>IIT</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr"/>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>Maskinteknik</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>Examensarbete i assisterande teknik med inriktning mot maskinteknik</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I111" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3K5</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>GMT3K6</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>MTA</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>IIT</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr"/>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>Maskinteknik</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
           <t>Forskningsmetodik för ingenjörer</t>
         </is>
       </c>
-      <c r="H104" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång</t>
-        </is>
-      </c>
-      <c r="I104" s="2" t="inlineStr">
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>Ingen aktiv kursomgång</t>
+        </is>
+      </c>
+      <c r="I112" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3K6</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I104"/>
+  <autoFilter ref="A1:I112"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I2" r:id="rId2"/>
@@ -5155,6 +5499,22 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I103" r:id="rId204"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A104" r:id="rId205"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I104" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A105" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I105" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A106" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I106" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A107" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I107" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A108" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I108" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A109" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I109" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A110" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I110" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A111" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I111" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A112" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I112" r:id="rId222"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update course descriptions and quality notes across various language programs
- Revised introductory lines for Chinese, Portuguese, Russian, Spanish, and Swedish to clarify subject areas.
- Updated course counts for Chinese and Swedish programs.
- Removed a course from the list of inactive course plans for Chinese.
- Adjusted tags and CSS classes for the Swedish course plan BSV22A.
- Added quality notes for multiple educational plans, highlighting discrepancies between program texts and course plan names, as well as listing any deprecated courses.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/01 IIT/Analys/Vilande kursplaner.xlsx
+++ b/vault-dalarna-university/01 IIT/Analys/Vilande kursplaner.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Vilande kursplaner" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Vilande kursplaner'!$A$1:$I$117</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Vilande kursplaner'!$A$1:$I$115</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I117"/>
+  <dimension ref="A1:I115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4089,12 +4089,12 @@
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>FEB222Q</t>
+          <t>GIK375</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>ENERGIBM</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -4110,12 +4110,12 @@
       <c r="E85" t="inlineStr"/>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Energisystem i byggd miljö</t>
+          <t>Informatik</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>Samarbetsprojekt inom energisystem</t>
+          <t>Komponentdriven webbdesign</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
@@ -4125,14 +4125,14 @@
       </c>
       <c r="I85" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FEB222Q</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK375</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>GIK375</t>
+          <t>GIK376</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -4158,7 +4158,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>Komponentdriven webbdesign</t>
+          <t>Applikationsutveckling för webben</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
@@ -4168,14 +4168,14 @@
       </c>
       <c r="I86" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK375</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK376</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>GIK376</t>
+          <t>GIK377</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -4201,7 +4201,7 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>Applikationsutveckling för webben</t>
+          <t>Utveckling av digitala tjänster</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
@@ -4211,14 +4211,14 @@
       </c>
       <c r="I87" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK376</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK377</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>GIK377</t>
+          <t>GIK38G</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -4233,7 +4233,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>2023-10-31</t>
+          <t>2023-12-19</t>
         </is>
       </c>
       <c r="E88" t="inlineStr"/>
@@ -4244,7 +4244,7 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>Utveckling av digitala tjänster</t>
+          <t>Design av digitala tjänster</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
@@ -4254,14 +4254,14 @@
       </c>
       <c r="I88" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK377</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK38G</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>GIK38G</t>
+          <t>GIK38H</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -4287,7 +4287,7 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>Design av digitala tjänster</t>
+          <t>Introduktion till IT och digitala tjänster</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
@@ -4297,14 +4297,14 @@
       </c>
       <c r="I89" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK38G</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK38H</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>GIK38H</t>
+          <t>GIK3BV</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -4319,7 +4319,7 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>2023-12-19</t>
+          <t>2024-05-23</t>
         </is>
       </c>
       <c r="E90" t="inlineStr"/>
@@ -4330,7 +4330,7 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>Introduktion till IT och digitala tjänster</t>
+          <t>E-samhället: e-förvaltning och digitala tjänster</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
@@ -4340,19 +4340,19 @@
       </c>
       <c r="I90" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK38H</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK3BV</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>GIK3BV</t>
+          <t>AEG2AY</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -4362,18 +4362,18 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>2024-05-23</t>
+          <t>2024-06-13</t>
         </is>
       </c>
       <c r="E91" t="inlineStr"/>
       <c r="F91" t="inlineStr">
         <is>
-          <t>Informatik</t>
+          <t>Energiteknik</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>E-samhället: e-förvaltning och digitala tjänster</t>
+          <t>Elektriska lagringssystem och tjänster</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
@@ -4383,14 +4383,14 @@
       </c>
       <c r="I91" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK3BV</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2AY</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>AEG2AY</t>
+          <t>AEG2B5</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -4416,7 +4416,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>Elektriska lagringssystem och tjänster</t>
+          <t>Projektkurs 3 - grupprojekt och kommunikation</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
@@ -4426,14 +4426,14 @@
       </c>
       <c r="I92" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2AY</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2B5</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>AEG2B5</t>
+          <t>AEG2AV</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -4448,7 +4448,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>2024-06-13</t>
+          <t>2024-12-12</t>
         </is>
       </c>
       <c r="E93" t="inlineStr"/>
@@ -4459,7 +4459,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>Projektkurs 3 - grupprojekt och kommunikation</t>
+          <t>Hållbarhet hos solenergisystem</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
@@ -4469,14 +4469,14 @@
       </c>
       <c r="I93" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2B5</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2AV</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>AEG2AV</t>
+          <t>AEG2AW</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -4502,7 +4502,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>Hållbarhet hos solenergisystem</t>
+          <t>Urbana energisystem</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
@@ -4512,14 +4512,14 @@
       </c>
       <c r="I94" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2AV</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2AW</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>AEG2AW</t>
+          <t>AEG2AX</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -4545,7 +4545,7 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>Urbana energisystem</t>
+          <t>Elnätsintegrering av förnybar kraft</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
@@ -4555,19 +4555,19 @@
       </c>
       <c r="I95" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2AW</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2AX</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>AEG2AX</t>
+          <t>GMD3FX</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -4577,18 +4577,18 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>2024-12-12</t>
+          <t>2025-05-22</t>
         </is>
       </c>
       <c r="E96" t="inlineStr"/>
       <c r="F96" t="inlineStr">
         <is>
-          <t>Energiteknik</t>
+          <t>Matematikdidaktik</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>Elnätsintegrering av förnybar kraft</t>
+          <t>Matematikutveckling i förskoleklass och årskurs 1–3 utifrån första- och andraspråksperspektiv</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
@@ -4598,19 +4598,19 @@
       </c>
       <c r="I96" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2AX</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD3FX</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>GMD3FX</t>
+          <t>GEG3FY</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -4626,12 +4626,12 @@
       <c r="E97" t="inlineStr"/>
       <c r="F97" t="inlineStr">
         <is>
-          <t>Matematikdidaktik</t>
+          <t>Energiteknik</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>Matematikutveckling i förskoleklass och årskurs 1–3 utifrån första- och andraspråksperspektiv</t>
+          <t>Praktik inom energiteknik</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
@@ -4641,19 +4641,19 @@
       </c>
       <c r="I97" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD3FX</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG3FY</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>GEG3FY</t>
+          <t>FDA222R</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>ANALYTIC</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -4663,18 +4663,18 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>2025-05-22</t>
+          <t>2025-09-17</t>
         </is>
       </c>
       <c r="E98" t="inlineStr"/>
       <c r="F98" t="inlineStr">
         <is>
-          <t>Energiteknik</t>
+          <t>Data Analytics</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>Praktik inom energiteknik</t>
+          <t>Komplexitet och operationsanalytiska metoder</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
@@ -4684,14 +4684,14 @@
       </c>
       <c r="I98" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG3FY</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FDA222R</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>FDA222R</t>
+          <t>FDA222S</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -4717,7 +4717,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>Komplexitet och operationsanalytiska metoder</t>
+          <t>Statistisk inlärning och maskininlärning</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
@@ -4727,14 +4727,14 @@
       </c>
       <c r="I99" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FDA222R</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FDA222S</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>FDA222S</t>
+          <t>FDA222T</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -4760,7 +4760,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>Statistisk inlärning och maskininlärning</t>
+          <t>Datadrivet beslutsfattande</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
@@ -4770,14 +4770,14 @@
       </c>
       <c r="I100" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FDA222S</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FDA222T</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>FDA222T</t>
+          <t>FDA222U</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -4803,7 +4803,7 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>Datadrivet beslutsfattande</t>
+          <t>Datainsamling och datakvalitet</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
@@ -4813,19 +4813,19 @@
       </c>
       <c r="I101" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FDA222T</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FDA222U</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>FDA222U</t>
+          <t>GMT3JQ</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>ANALYTIC</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -4835,18 +4835,18 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>2025-09-17</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="E102" t="inlineStr"/>
       <c r="F102" t="inlineStr">
         <is>
-          <t>Data Analytics</t>
+          <t>Maskinteknik</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>Datainsamling och datakvalitet</t>
+          <t>Mekatronik</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
@@ -4856,14 +4856,14 @@
       </c>
       <c r="I102" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FDA222U</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3JQ</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>GMT3JQ</t>
+          <t>GMT3JR</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -4889,7 +4889,7 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>Mekatronik</t>
+          <t>Termodynamik</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
@@ -4899,14 +4899,14 @@
       </c>
       <c r="I103" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3JQ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3JR</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>GMT3JR</t>
+          <t>GMT3JY</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -4932,7 +4932,7 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>Termodynamik</t>
+          <t>Tillverkning</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
@@ -4942,19 +4942,19 @@
       </c>
       <c r="I104" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3JR</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3JY</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>GMT3JY</t>
+          <t>GIE3JW</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>IEA</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -4964,18 +4964,18 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="E105" t="inlineStr"/>
       <c r="F105" t="inlineStr">
         <is>
-          <t>Maskinteknik</t>
+          <t>Industriell ekonomi</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>Tillverkning</t>
+          <t>Innovation och entreprenörskap inom assisterande teknik</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
@@ -4985,19 +4985,19 @@
       </c>
       <c r="I105" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3JY</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE3JW</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>GIE3JW</t>
+          <t>GMT3JT</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>IEA</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -5013,12 +5013,12 @@
       <c r="E106" t="inlineStr"/>
       <c r="F106" t="inlineStr">
         <is>
-          <t>Industriell ekonomi</t>
+          <t>Maskinteknik</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>Innovation och entreprenörskap inom assisterande teknik</t>
+          <t>Tillämpning av regelverk för assisterande produkter</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
@@ -5028,14 +5028,14 @@
       </c>
       <c r="I106" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE3JW</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3JT</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>GMT3JT</t>
+          <t>GMT3JU</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -5061,7 +5061,7 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>Tillämpning av regelverk för assisterande produkter</t>
+          <t>Smarta hem och e-hälsoteknik</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
@@ -5071,14 +5071,14 @@
       </c>
       <c r="I107" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3JT</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3JU</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>GMT3JU</t>
+          <t>GMT3JV</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -5104,7 +5104,7 @@
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>Smarta hem och e-hälsoteknik</t>
+          <t>Assisterande robotik</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
@@ -5114,19 +5114,19 @@
       </c>
       <c r="I108" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3JU</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3JV</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>GMT3JV</t>
+          <t>BMA228</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>MAA</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -5136,18 +5136,18 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="E109" t="inlineStr"/>
       <c r="F109" t="inlineStr">
         <is>
-          <t>Maskinteknik</t>
+          <t>Matematik</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>Assisterande robotik</t>
+          <t>Basmatematik 1</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
@@ -5157,14 +5157,14 @@
       </c>
       <c r="I109" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3JV</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BMA228</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>BMA228</t>
+          <t>BMA229</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -5190,7 +5190,7 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>Basmatematik 1</t>
+          <t>Basmatematik 2</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
@@ -5200,19 +5200,19 @@
       </c>
       <c r="I110" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BMA228</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BMA229</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>BMA229</t>
+          <t>GMT3K5</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>MAA</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -5228,12 +5228,12 @@
       <c r="E111" t="inlineStr"/>
       <c r="F111" t="inlineStr">
         <is>
-          <t>Matematik</t>
+          <t>Maskinteknik</t>
         </is>
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>Basmatematik 2</t>
+          <t>Examensarbete i assisterande teknik med inriktning mot maskinteknik</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
@@ -5243,14 +5243,14 @@
       </c>
       <c r="I111" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BMA229</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3K5</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>GMT3K5</t>
+          <t>GMT3K6</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -5276,7 +5276,7 @@
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>Examensarbete i assisterande teknik med inriktning mot maskinteknik</t>
+          <t>Forskningsmetodik för ingenjörer</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">
@@ -5286,19 +5286,19 @@
       </c>
       <c r="I112" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3K5</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3K6</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>GMT3K6</t>
+          <t>GDV3KX</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>DVE</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -5308,18 +5308,18 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="E113" t="inlineStr"/>
       <c r="F113" t="inlineStr">
         <is>
-          <t>Maskinteknik</t>
+          <t>Datavetenskaper</t>
         </is>
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>Forskningsmetodik för ingenjörer</t>
+          <t>Programutvecklingsteknik</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
@@ -5329,14 +5329,14 @@
       </c>
       <c r="I113" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3K6</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GDV3KX</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>GDV3KW</t>
+          <t>GDV3KY</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -5362,7 +5362,7 @@
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>Relationsdatabaser</t>
+          <t>Datasäkerhet och integritet</t>
         </is>
       </c>
       <c r="H114" t="inlineStr">
@@ -5372,14 +5372,14 @@
       </c>
       <c r="I114" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GDV3KW</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GDV3KY</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>GDV3KX</t>
+          <t>GDV3KZ</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -5405,7 +5405,7 @@
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>Programutvecklingsteknik</t>
+          <t>Projekt och agila arbetsmetoder</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">
@@ -5415,98 +5415,12 @@
       </c>
       <c r="I115" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GDV3KX</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" s="2" t="inlineStr">
-        <is>
-          <t>GDV3KY</t>
-        </is>
-      </c>
-      <c r="B116" t="inlineStr">
-        <is>
-          <t>DVE</t>
-        </is>
-      </c>
-      <c r="C116" t="inlineStr">
-        <is>
-          <t>IIT</t>
-        </is>
-      </c>
-      <c r="D116" t="inlineStr">
-        <is>
-          <t>2026-06-23</t>
-        </is>
-      </c>
-      <c r="E116" t="inlineStr"/>
-      <c r="F116" t="inlineStr">
-        <is>
-          <t>Datavetenskaper</t>
-        </is>
-      </c>
-      <c r="G116" t="inlineStr">
-        <is>
-          <t>Datasäkerhet och integritet</t>
-        </is>
-      </c>
-      <c r="H116" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång</t>
-        </is>
-      </c>
-      <c r="I116" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GDV3KY</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" s="2" t="inlineStr">
-        <is>
-          <t>GDV3KZ</t>
-        </is>
-      </c>
-      <c r="B117" t="inlineStr">
-        <is>
-          <t>DVE</t>
-        </is>
-      </c>
-      <c r="C117" t="inlineStr">
-        <is>
-          <t>IIT</t>
-        </is>
-      </c>
-      <c r="D117" t="inlineStr">
-        <is>
-          <t>2026-06-23</t>
-        </is>
-      </c>
-      <c r="E117" t="inlineStr"/>
-      <c r="F117" t="inlineStr">
-        <is>
-          <t>Datavetenskaper</t>
-        </is>
-      </c>
-      <c r="G117" t="inlineStr">
-        <is>
-          <t>Projekt och agila arbetsmetoder</t>
-        </is>
-      </c>
-      <c r="H117" t="inlineStr">
-        <is>
-          <t>Ingen aktiv kursomgång</t>
-        </is>
-      </c>
-      <c r="I117" s="2" t="inlineStr">
-        <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GDV3KZ</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I117"/>
+  <autoFilter ref="A1:I115"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I2" r:id="rId2"/>
@@ -5736,10 +5650,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I114" r:id="rId226"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A115" r:id="rId227"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I115" r:id="rId228"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A116" r:id="rId229"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I116" r:id="rId230"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A117" r:id="rId231"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I117" r:id="rId232"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>